<commit_message>
fix: Populate discount_percent_str, discount_price, discount_price_per_sq_ft and payment_method for 叡璟I unit popover cards
</commit_message>
<xml_diff>
--- a/files/九龙-深水埗-叡璟I.xlsx
+++ b/files/九龙-深水埗-叡璟I.xlsx
@@ -651,7 +651,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -4786,22 +4786,18 @@
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K62" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L62" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K62" s="5" t="n">
+        <v>12370680</v>
+      </c>
+      <c r="L62" s="5" t="n">
+        <v>18829</v>
       </c>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N62" s="3" t="inlineStr">
@@ -5190,22 +5186,18 @@
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K68" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L68" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K68" s="5" t="n">
+        <v>12333720</v>
+      </c>
+      <c r="L68" s="5" t="n">
+        <v>18773</v>
       </c>
       <c r="M68" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N68" s="3" t="inlineStr">
@@ -5594,22 +5586,18 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K74" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L74" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="n">
+        <v>12296760</v>
+      </c>
+      <c r="L74" s="5" t="n">
+        <v>18717</v>
       </c>
       <c r="M74" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N74" s="3" t="inlineStr">
@@ -5998,22 +5986,18 @@
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K80" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L80" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="n">
+        <v>12259800</v>
+      </c>
+      <c r="L80" s="5" t="n">
+        <v>18660</v>
       </c>
       <c r="M80" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N80" s="3" t="inlineStr">
@@ -6402,22 +6386,18 @@
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K86" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L86" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K86" s="5" t="n">
+        <v>12223680</v>
+      </c>
+      <c r="L86" s="5" t="n">
+        <v>18605</v>
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N86" s="3" t="inlineStr">
@@ -6806,22 +6786,18 @@
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K92" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L92" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K92" s="5" t="n">
+        <v>12186720</v>
+      </c>
+      <c r="L92" s="5" t="n">
+        <v>18549</v>
       </c>
       <c r="M92" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N92" s="3" t="inlineStr">
@@ -7210,22 +7186,18 @@
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K98" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L98" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K98" s="5" t="n">
+        <v>12150600</v>
+      </c>
+      <c r="L98" s="5" t="n">
+        <v>18494</v>
       </c>
       <c r="M98" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N98" s="3" t="inlineStr">
@@ -7614,22 +7586,18 @@
       </c>
       <c r="J104" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K104" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L104" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K104" s="5" t="n">
+        <v>12150600</v>
+      </c>
+      <c r="L104" s="5" t="n">
+        <v>18494</v>
       </c>
       <c r="M104" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N104" s="3" t="inlineStr">
@@ -8018,22 +7986,18 @@
       </c>
       <c r="J110" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K110" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L110" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K110" s="5" t="n">
+        <v>12078360</v>
+      </c>
+      <c r="L110" s="5" t="n">
+        <v>18384</v>
       </c>
       <c r="M110" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N110" s="3" t="inlineStr">
@@ -10054,22 +10018,18 @@
       </c>
       <c r="J140" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K140" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L140" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K140" s="5" t="n">
+        <v>11922120</v>
+      </c>
+      <c r="L140" s="5" t="n">
+        <v>18146</v>
       </c>
       <c r="M140" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N140" s="3" t="inlineStr">
@@ -10458,22 +10418,18 @@
       </c>
       <c r="J146" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K146" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L146" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K146" s="5" t="n">
+        <v>11897760</v>
+      </c>
+      <c r="L146" s="5" t="n">
+        <v>18109</v>
       </c>
       <c r="M146" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N146" s="3" t="inlineStr">
@@ -10862,22 +10818,18 @@
       </c>
       <c r="J152" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K152" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L152" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K152" s="5" t="n">
+        <v>11874240</v>
+      </c>
+      <c r="L152" s="5" t="n">
+        <v>18073</v>
       </c>
       <c r="M152" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N152" s="3" t="inlineStr">
@@ -11402,22 +11354,18 @@
       </c>
       <c r="J160" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K160" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L160" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K160" s="5" t="n">
+        <v>7568400</v>
+      </c>
+      <c r="L160" s="5" t="n">
+        <v>17935</v>
       </c>
       <c r="M160" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N160" s="3" t="inlineStr">
@@ -11806,22 +11754,18 @@
       </c>
       <c r="J166" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K166" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L166" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K166" s="5" t="n">
+        <v>7545720</v>
+      </c>
+      <c r="L166" s="5" t="n">
+        <v>17881</v>
       </c>
       <c r="M166" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N166" s="3" t="inlineStr">
@@ -12210,22 +12154,18 @@
       </c>
       <c r="J172" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K172" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L172" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K172" s="5" t="n">
+        <v>7523040</v>
+      </c>
+      <c r="L172" s="5" t="n">
+        <v>17827</v>
       </c>
       <c r="M172" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N172" s="3" t="inlineStr">
@@ -12478,22 +12418,18 @@
       </c>
       <c r="J176" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K176" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L176" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K176" s="5" t="n">
+        <v>11779320</v>
+      </c>
+      <c r="L176" s="5" t="n">
+        <v>17929</v>
       </c>
       <c r="M176" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N176" s="3" t="inlineStr">
@@ -12610,22 +12546,18 @@
       </c>
       <c r="J178" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K178" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L178" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K178" s="5" t="n">
+        <v>7485240</v>
+      </c>
+      <c r="L178" s="5" t="n">
+        <v>17738</v>
       </c>
       <c r="M178" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N178" s="3" t="inlineStr">
@@ -12878,22 +12810,18 @@
       </c>
       <c r="J182" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K182" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L182" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K182" s="5" t="n">
+        <v>11755800</v>
+      </c>
+      <c r="L182" s="5" t="n">
+        <v>17893</v>
       </c>
       <c r="M182" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N182" s="3" t="inlineStr">
@@ -13010,22 +12938,18 @@
       </c>
       <c r="J184" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K184" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L184" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K184" s="5" t="n">
+        <v>7433160</v>
+      </c>
+      <c r="L184" s="5" t="n">
+        <v>17614</v>
       </c>
       <c r="M184" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N184" s="3" t="inlineStr">
@@ -13278,22 +13202,18 @@
       </c>
       <c r="J188" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K188" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L188" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K188" s="5" t="n">
+        <v>11732280</v>
+      </c>
+      <c r="L188" s="5" t="n">
+        <v>17857</v>
       </c>
       <c r="M188" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N188" s="3" t="inlineStr">
@@ -13410,22 +13330,18 @@
       </c>
       <c r="J190" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K190" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L190" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K190" s="5" t="n">
+        <v>7321440</v>
+      </c>
+      <c r="L190" s="5" t="n">
+        <v>17349</v>
       </c>
       <c r="M190" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N190" s="3" t="inlineStr">
@@ -13814,22 +13730,18 @@
       </c>
       <c r="J196" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K196" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L196" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K196" s="5" t="n">
+        <v>7138320</v>
+      </c>
+      <c r="L196" s="5" t="n">
+        <v>16915</v>
       </c>
       <c r="M196" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N196" s="3" t="inlineStr">
@@ -14218,22 +14130,18 @@
       </c>
       <c r="J202" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K202" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L202" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K202" s="5" t="n">
+        <v>7138320</v>
+      </c>
+      <c r="L202" s="5" t="n">
+        <v>16915</v>
       </c>
       <c r="M202" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N202" s="3" t="inlineStr">
@@ -14622,22 +14530,18 @@
       </c>
       <c r="J208" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K208" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L208" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K208" s="5" t="n">
+        <v>7095480</v>
+      </c>
+      <c r="L208" s="5" t="n">
+        <v>16814</v>
       </c>
       <c r="M208" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N208" s="3" t="inlineStr">
@@ -14890,22 +14794,18 @@
       </c>
       <c r="J212" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K212" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L212" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K212" s="5" t="n">
+        <v>11639040</v>
+      </c>
+      <c r="L212" s="5" t="n">
+        <v>17715</v>
       </c>
       <c r="M212" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N212" s="3" t="inlineStr">
@@ -15022,22 +14922,18 @@
       </c>
       <c r="J214" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K214" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L214" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K214" s="5" t="n">
+        <v>7074480</v>
+      </c>
+      <c r="L214" s="5" t="n">
+        <v>16764</v>
       </c>
       <c r="M214" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N214" s="3" t="inlineStr">
@@ -15290,22 +15186,18 @@
       </c>
       <c r="J218" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K218" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L218" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K218" s="5" t="n">
+        <v>11615520</v>
+      </c>
+      <c r="L218" s="5" t="n">
+        <v>17680</v>
       </c>
       <c r="M218" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N218" s="3" t="inlineStr">
@@ -15422,22 +15314,18 @@
       </c>
       <c r="J220" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K220" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L220" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K220" s="5" t="n">
+        <v>7032480</v>
+      </c>
+      <c r="L220" s="5" t="n">
+        <v>16665</v>
       </c>
       <c r="M220" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N220" s="3" t="inlineStr">
@@ -15690,22 +15578,18 @@
       </c>
       <c r="J224" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K224" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L224" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K224" s="5" t="n">
+        <v>11607120</v>
+      </c>
+      <c r="L224" s="5" t="n">
+        <v>17667</v>
       </c>
       <c r="M224" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N224" s="3" t="inlineStr">
@@ -16162,22 +16046,18 @@
       </c>
       <c r="J231" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K231" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L231" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K231" s="5" t="n">
+        <v>7830480</v>
+      </c>
+      <c r="L231" s="5" t="n">
+        <v>18733</v>
       </c>
       <c r="M231" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N231" s="3" t="inlineStr">
@@ -16226,22 +16106,18 @@
       </c>
       <c r="J232" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K232" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L232" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K232" s="5" t="n">
+        <v>7807800</v>
+      </c>
+      <c r="L232" s="5" t="n">
+        <v>18679</v>
       </c>
       <c r="M232" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N232" s="3" t="inlineStr">
@@ -16290,22 +16166,18 @@
       </c>
       <c r="J233" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K233" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L233" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K233" s="5" t="n">
+        <v>7784280</v>
+      </c>
+      <c r="L233" s="5" t="n">
+        <v>18623</v>
       </c>
       <c r="M233" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N233" s="3" t="inlineStr">
@@ -16830,22 +16702,18 @@
       </c>
       <c r="J241" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K241" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L241" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K241" s="5" t="n">
+        <v>7760760</v>
+      </c>
+      <c r="L241" s="5" t="n">
+        <v>18566</v>
       </c>
       <c r="M241" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N241" s="3" t="inlineStr">
@@ -17370,22 +17238,18 @@
       </c>
       <c r="J249" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K249" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L249" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K249" s="5" t="n">
+        <v>7737240</v>
+      </c>
+      <c r="L249" s="5" t="n">
+        <v>18510</v>
       </c>
       <c r="M249" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N249" s="3" t="inlineStr">
@@ -17910,22 +17774,18 @@
       </c>
       <c r="J257" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K257" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L257" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K257" s="5" t="n">
+        <v>7714560</v>
+      </c>
+      <c r="L257" s="5" t="n">
+        <v>18456</v>
       </c>
       <c r="M257" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N257" s="3" t="inlineStr">
@@ -18450,22 +18310,18 @@
       </c>
       <c r="J265" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K265" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L265" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K265" s="5" t="n">
+        <v>7714560</v>
+      </c>
+      <c r="L265" s="5" t="n">
+        <v>18456</v>
       </c>
       <c r="M265" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N265" s="3" t="inlineStr">
@@ -18990,22 +18846,18 @@
       </c>
       <c r="J273" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K273" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L273" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K273" s="5" t="n">
+        <v>7668360</v>
+      </c>
+      <c r="L273" s="5" t="n">
+        <v>18345</v>
       </c>
       <c r="M273" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N273" s="3" t="inlineStr">
@@ -19530,22 +19382,18 @@
       </c>
       <c r="J281" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K281" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L281" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K281" s="5" t="n">
+        <v>7645680</v>
+      </c>
+      <c r="L281" s="5" t="n">
+        <v>18291</v>
       </c>
       <c r="M281" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N281" s="3" t="inlineStr">
@@ -19662,22 +19510,18 @@
       </c>
       <c r="J283" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K283" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L283" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K283" s="5" t="n">
+        <v>5902680</v>
+      </c>
+      <c r="L283" s="5" t="n">
+        <v>19290</v>
       </c>
       <c r="M283" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N283" s="3" t="inlineStr">
@@ -20066,22 +19910,18 @@
       </c>
       <c r="J289" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K289" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L289" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K289" s="5" t="n">
+        <v>7623000</v>
+      </c>
+      <c r="L289" s="5" t="n">
+        <v>18237</v>
       </c>
       <c r="M289" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N289" s="3" t="inlineStr">
@@ -20198,22 +20038,18 @@
       </c>
       <c r="J291" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K291" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L291" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K291" s="5" t="n">
+        <v>5885040</v>
+      </c>
+      <c r="L291" s="5" t="n">
+        <v>19232</v>
       </c>
       <c r="M291" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N291" s="3" t="inlineStr">
@@ -20602,22 +20438,18 @@
       </c>
       <c r="J297" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K297" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L297" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K297" s="5" t="n">
+        <v>7599480</v>
+      </c>
+      <c r="L297" s="5" t="n">
+        <v>18181</v>
       </c>
       <c r="M297" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N297" s="3" t="inlineStr">
@@ -20734,22 +20566,18 @@
       </c>
       <c r="J299" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K299" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L299" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K299" s="5" t="n">
+        <v>5867400</v>
+      </c>
+      <c r="L299" s="5" t="n">
+        <v>19175</v>
       </c>
       <c r="M299" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N299" s="3" t="inlineStr">
@@ -21138,22 +20966,18 @@
       </c>
       <c r="J305" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K305" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L305" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K305" s="5" t="n">
+        <v>7576800</v>
+      </c>
+      <c r="L305" s="5" t="n">
+        <v>18126</v>
       </c>
       <c r="M305" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N305" s="3" t="inlineStr">
@@ -21270,22 +21094,18 @@
       </c>
       <c r="J307" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K307" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L307" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K307" s="5" t="n">
+        <v>5849760</v>
+      </c>
+      <c r="L307" s="5" t="n">
+        <v>19117</v>
       </c>
       <c r="M307" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N307" s="3" t="inlineStr">
@@ -21674,22 +21494,18 @@
       </c>
       <c r="J313" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K313" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L313" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K313" s="5" t="n">
+        <v>7554120</v>
+      </c>
+      <c r="L313" s="5" t="n">
+        <v>18072</v>
       </c>
       <c r="M313" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N313" s="3" t="inlineStr">
@@ -21806,22 +21622,18 @@
       </c>
       <c r="J315" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K315" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L315" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K315" s="5" t="n">
+        <v>5832120</v>
+      </c>
+      <c r="L315" s="5" t="n">
+        <v>19059</v>
       </c>
       <c r="M315" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N315" s="3" t="inlineStr">
@@ -22210,22 +22022,18 @@
       </c>
       <c r="J321" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K321" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L321" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K321" s="5" t="n">
+        <v>7531440</v>
+      </c>
+      <c r="L321" s="5" t="n">
+        <v>18018</v>
       </c>
       <c r="M321" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N321" s="3" t="inlineStr">
@@ -22342,22 +22150,18 @@
       </c>
       <c r="J323" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K323" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L323" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K323" s="5" t="n">
+        <v>5814480</v>
+      </c>
+      <c r="L323" s="5" t="n">
+        <v>19002</v>
       </c>
       <c r="M323" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N323" s="3" t="inlineStr">
@@ -22746,22 +22550,18 @@
       </c>
       <c r="J329" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K329" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L329" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K329" s="5" t="n">
+        <v>7509600</v>
+      </c>
+      <c r="L329" s="5" t="n">
+        <v>17966</v>
       </c>
       <c r="M329" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N329" s="3" t="inlineStr">
@@ -22878,22 +22678,18 @@
       </c>
       <c r="J331" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K331" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L331" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K331" s="5" t="n">
+        <v>5797680</v>
+      </c>
+      <c r="L331" s="5" t="n">
+        <v>18947</v>
       </c>
       <c r="M331" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N331" s="3" t="inlineStr">
@@ -23282,22 +23078,18 @@
       </c>
       <c r="J337" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K337" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L337" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K337" s="5" t="n">
+        <v>7509600</v>
+      </c>
+      <c r="L337" s="5" t="n">
+        <v>17966</v>
       </c>
       <c r="M337" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N337" s="3" t="inlineStr">
@@ -23414,22 +23206,18 @@
       </c>
       <c r="J339" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K339" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L339" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K339" s="5" t="n">
+        <v>5797680</v>
+      </c>
+      <c r="L339" s="5" t="n">
+        <v>18947</v>
       </c>
       <c r="M339" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N339" s="3" t="inlineStr">
@@ -23818,22 +23606,18 @@
       </c>
       <c r="J345" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K345" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L345" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K345" s="5" t="n">
+        <v>7464240</v>
+      </c>
+      <c r="L345" s="5" t="n">
+        <v>17857</v>
       </c>
       <c r="M345" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N345" s="3" t="inlineStr">
@@ -23950,22 +23734,18 @@
       </c>
       <c r="J347" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K347" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L347" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K347" s="5" t="n">
+        <v>5763240</v>
+      </c>
+      <c r="L347" s="5" t="n">
+        <v>18834</v>
       </c>
       <c r="M347" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N347" s="3" t="inlineStr">
@@ -24354,22 +24134,18 @@
       </c>
       <c r="J353" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K353" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L353" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K353" s="5" t="n">
+        <v>7460880</v>
+      </c>
+      <c r="L353" s="5" t="n">
+        <v>17849</v>
       </c>
       <c r="M353" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N353" s="3" t="inlineStr">
@@ -24894,22 +24670,18 @@
       </c>
       <c r="J361" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K361" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L361" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K361" s="5" t="n">
+        <v>7445760</v>
+      </c>
+      <c r="L361" s="5" t="n">
+        <v>17813</v>
       </c>
       <c r="M361" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N361" s="3" t="inlineStr">
@@ -25978,22 +25750,18 @@
       </c>
       <c r="J377" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K377" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L377" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K377" s="5" t="n">
+        <v>7430640</v>
+      </c>
+      <c r="L377" s="5" t="n">
+        <v>17777</v>
       </c>
       <c r="M377" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N377" s="3" t="inlineStr">
@@ -26314,22 +26082,18 @@
       </c>
       <c r="J382" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K382" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L382" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K382" s="5" t="n">
+        <v>8657040</v>
+      </c>
+      <c r="L382" s="5" t="n">
+        <v>18187</v>
       </c>
       <c r="M382" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N382" s="3" t="inlineStr">
@@ -26514,22 +26278,18 @@
       </c>
       <c r="J385" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K385" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L385" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K385" s="5" t="n">
+        <v>7415520</v>
+      </c>
+      <c r="L385" s="5" t="n">
+        <v>17740</v>
       </c>
       <c r="M385" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N385" s="3" t="inlineStr">
@@ -26646,22 +26406,18 @@
       </c>
       <c r="J387" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K387" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L387" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K387" s="5" t="n">
+        <v>5617080</v>
+      </c>
+      <c r="L387" s="5" t="n">
+        <v>18356</v>
       </c>
       <c r="M387" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N387" s="3" t="inlineStr">
@@ -26846,22 +26602,18 @@
       </c>
       <c r="J390" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K390" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L390" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K390" s="5" t="n">
+        <v>8631000</v>
+      </c>
+      <c r="L390" s="5" t="n">
+        <v>18132</v>
       </c>
       <c r="M390" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N390" s="3" t="inlineStr">
@@ -27046,22 +26798,18 @@
       </c>
       <c r="J393" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K393" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L393" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K393" s="5" t="n">
+        <v>7401240</v>
+      </c>
+      <c r="L393" s="5" t="n">
+        <v>17706</v>
       </c>
       <c r="M393" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N393" s="3" t="inlineStr">
@@ -27178,22 +26926,18 @@
       </c>
       <c r="J395" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K395" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L395" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K395" s="5" t="n">
+        <v>5600280</v>
+      </c>
+      <c r="L395" s="5" t="n">
+        <v>18302</v>
       </c>
       <c r="M395" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N395" s="3" t="inlineStr">
@@ -27378,22 +27122,18 @@
       </c>
       <c r="J398" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K398" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L398" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K398" s="5" t="n">
+        <v>8604960</v>
+      </c>
+      <c r="L398" s="5" t="n">
+        <v>18078</v>
       </c>
       <c r="M398" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N398" s="3" t="inlineStr">
@@ -27578,22 +27318,18 @@
       </c>
       <c r="J401" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K401" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L401" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K401" s="5" t="n">
+        <v>7386120</v>
+      </c>
+      <c r="L401" s="5" t="n">
+        <v>17670</v>
       </c>
       <c r="M401" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N401" s="3" t="inlineStr">
@@ -27710,22 +27446,18 @@
       </c>
       <c r="J403" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K403" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L403" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K403" s="5" t="n">
+        <v>5583480</v>
+      </c>
+      <c r="L403" s="5" t="n">
+        <v>18247</v>
       </c>
       <c r="M403" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N403" s="3" t="inlineStr">
@@ -28114,22 +27846,18 @@
       </c>
       <c r="J409" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K409" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L409" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K409" s="5" t="n">
+        <v>7386120</v>
+      </c>
+      <c r="L409" s="5" t="n">
+        <v>17670</v>
       </c>
       <c r="M409" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N409" s="3" t="inlineStr">
@@ -28586,22 +28314,18 @@
       </c>
       <c r="J416" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K416" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L416" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K416" s="5" t="n">
+        <v>7974960</v>
+      </c>
+      <c r="L416" s="5" t="n">
+        <v>17801</v>
       </c>
       <c r="M416" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N416" s="3" t="inlineStr">
@@ -28650,22 +28374,18 @@
       </c>
       <c r="J417" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K417" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L417" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K417" s="5" t="n">
+        <v>7356720</v>
+      </c>
+      <c r="L417" s="5" t="n">
+        <v>17600</v>
       </c>
       <c r="M417" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N417" s="3" t="inlineStr">
@@ -29122,22 +28842,18 @@
       </c>
       <c r="J424" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K424" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L424" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K424" s="5" t="n">
+        <v>7951440</v>
+      </c>
+      <c r="L424" s="5" t="n">
+        <v>17749</v>
       </c>
       <c r="M424" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N424" s="3" t="inlineStr">
@@ -29186,22 +28902,18 @@
       </c>
       <c r="J425" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K425" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L425" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K425" s="5" t="n">
+        <v>7342440</v>
+      </c>
+      <c r="L425" s="5" t="n">
+        <v>17566</v>
       </c>
       <c r="M425" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N425" s="3" t="inlineStr">
@@ -29522,22 +29234,18 @@
       </c>
       <c r="J430" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K430" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L430" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K430" s="5" t="n">
+        <v>8502480</v>
+      </c>
+      <c r="L430" s="5" t="n">
+        <v>17862</v>
       </c>
       <c r="M430" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N430" s="3" t="inlineStr">
@@ -29654,22 +29362,18 @@
       </c>
       <c r="J432" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K432" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L432" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K432" s="5" t="n">
+        <v>7927920</v>
+      </c>
+      <c r="L432" s="5" t="n">
+        <v>17696</v>
       </c>
       <c r="M432" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N432" s="3" t="inlineStr">
@@ -29718,22 +29422,18 @@
       </c>
       <c r="J433" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K433" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L433" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K433" s="5" t="n">
+        <v>7327320</v>
+      </c>
+      <c r="L433" s="5" t="n">
+        <v>17529</v>
       </c>
       <c r="M433" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N433" s="3" t="inlineStr">
@@ -29850,22 +29550,18 @@
       </c>
       <c r="J435" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K435" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L435" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K435" s="5" t="n">
+        <v>5516280</v>
+      </c>
+      <c r="L435" s="5" t="n">
+        <v>18027</v>
       </c>
       <c r="M435" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N435" s="3" t="inlineStr">
@@ -30050,22 +29746,18 @@
       </c>
       <c r="J438" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K438" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L438" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K438" s="5" t="n">
+        <v>8459640</v>
+      </c>
+      <c r="L438" s="5" t="n">
+        <v>17772</v>
       </c>
       <c r="M438" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N438" s="3" t="inlineStr">
@@ -30182,22 +29874,18 @@
       </c>
       <c r="J440" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K440" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L440" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K440" s="5" t="n">
+        <v>7887600</v>
+      </c>
+      <c r="L440" s="5" t="n">
+        <v>17606</v>
       </c>
       <c r="M440" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N440" s="3" t="inlineStr">
@@ -30246,22 +29934,18 @@
       </c>
       <c r="J441" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K441" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L441" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K441" s="5" t="n">
+        <v>7313040</v>
+      </c>
+      <c r="L441" s="5" t="n">
+        <v>17495</v>
       </c>
       <c r="M441" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N441" s="3" t="inlineStr">
@@ -30378,22 +30062,18 @@
       </c>
       <c r="J443" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K443" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L443" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K443" s="5" t="n">
+        <v>5500320</v>
+      </c>
+      <c r="L443" s="5" t="n">
+        <v>17975</v>
       </c>
       <c r="M443" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N443" s="3" t="inlineStr">
@@ -30578,22 +30258,18 @@
       </c>
       <c r="J446" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K446" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L446" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K446" s="5" t="n">
+        <v>8400840</v>
+      </c>
+      <c r="L446" s="5" t="n">
+        <v>17649</v>
       </c>
       <c r="M446" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N446" s="3" t="inlineStr">
@@ -30710,22 +30386,18 @@
       </c>
       <c r="J448" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K448" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L448" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K448" s="5" t="n">
+        <v>7833000</v>
+      </c>
+      <c r="L448" s="5" t="n">
+        <v>17484</v>
       </c>
       <c r="M448" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N448" s="3" t="inlineStr">
@@ -30774,22 +30446,18 @@
       </c>
       <c r="J449" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K449" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L449" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K449" s="5" t="n">
+        <v>7297920</v>
+      </c>
+      <c r="L449" s="5" t="n">
+        <v>17459</v>
       </c>
       <c r="M449" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N449" s="3" t="inlineStr">
@@ -30906,22 +30574,18 @@
       </c>
       <c r="J451" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K451" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L451" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K451" s="5" t="n">
+        <v>5483520</v>
+      </c>
+      <c r="L451" s="5" t="n">
+        <v>17920</v>
       </c>
       <c r="M451" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N451" s="3" t="inlineStr">
@@ -31242,22 +30906,18 @@
       </c>
       <c r="J456" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K456" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L456" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K456" s="5" t="n">
+        <v>7715400</v>
+      </c>
+      <c r="L456" s="5" t="n">
+        <v>17222</v>
       </c>
       <c r="M456" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N456" s="3" t="inlineStr">
@@ -31306,22 +30966,18 @@
       </c>
       <c r="J457" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K457" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L457" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K457" s="5" t="n">
+        <v>7283640</v>
+      </c>
+      <c r="L457" s="5" t="n">
+        <v>17425</v>
       </c>
       <c r="M457" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N457" s="3" t="inlineStr">
@@ -31778,22 +31434,18 @@
       </c>
       <c r="J464" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K464" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L464" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K464" s="5" t="n">
+        <v>7522200</v>
+      </c>
+      <c r="L464" s="5" t="n">
+        <v>16791</v>
       </c>
       <c r="M464" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N464" s="3" t="inlineStr">
@@ -31842,22 +31494,18 @@
       </c>
       <c r="J465" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K465" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L465" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K465" s="5" t="n">
+        <v>7268520</v>
+      </c>
+      <c r="L465" s="5" t="n">
+        <v>17389</v>
       </c>
       <c r="M465" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N465" s="3" t="inlineStr">
@@ -32314,22 +31962,18 @@
       </c>
       <c r="J472" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K472" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L472" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K472" s="5" t="n">
+        <v>7522200</v>
+      </c>
+      <c r="L472" s="5" t="n">
+        <v>16791</v>
       </c>
       <c r="M472" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N472" s="3" t="inlineStr">
@@ -32378,22 +32022,18 @@
       </c>
       <c r="J473" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K473" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L473" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K473" s="5" t="n">
+        <v>7268520</v>
+      </c>
+      <c r="L473" s="5" t="n">
+        <v>17389</v>
       </c>
       <c r="M473" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N473" s="3" t="inlineStr">
@@ -32714,22 +32354,18 @@
       </c>
       <c r="J478" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K478" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L478" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K478" s="5" t="n">
+        <v>8019480</v>
+      </c>
+      <c r="L478" s="5" t="n">
+        <v>16848</v>
       </c>
       <c r="M478" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N478" s="3" t="inlineStr">
@@ -32846,22 +32482,18 @@
       </c>
       <c r="J480" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K480" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L480" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K480" s="5" t="n">
+        <v>7476840</v>
+      </c>
+      <c r="L480" s="5" t="n">
+        <v>16689</v>
       </c>
       <c r="M480" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N480" s="3" t="inlineStr">
@@ -32910,22 +32542,18 @@
       </c>
       <c r="J481" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K481" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L481" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K481" s="5" t="n">
+        <v>7239960</v>
+      </c>
+      <c r="L481" s="5" t="n">
+        <v>17320</v>
       </c>
       <c r="M481" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N481" s="3" t="inlineStr">
@@ -33042,22 +32670,18 @@
       </c>
       <c r="J483" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K483" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L483" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K483" s="5" t="n">
+        <v>5418000</v>
+      </c>
+      <c r="L483" s="5" t="n">
+        <v>17706</v>
       </c>
       <c r="M483" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N483" s="3" t="inlineStr">
@@ -33242,22 +32866,18 @@
       </c>
       <c r="J486" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K486" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L486" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K486" s="5" t="n">
+        <v>7995120</v>
+      </c>
+      <c r="L486" s="5" t="n">
+        <v>16796</v>
       </c>
       <c r="M486" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N486" s="3" t="inlineStr">
@@ -33374,22 +32994,18 @@
       </c>
       <c r="J488" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K488" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L488" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K488" s="5" t="n">
+        <v>7455000</v>
+      </c>
+      <c r="L488" s="5" t="n">
+        <v>16641</v>
       </c>
       <c r="M488" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N488" s="3" t="inlineStr">
@@ -33438,22 +33054,18 @@
       </c>
       <c r="J489" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K489" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L489" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K489" s="5" t="n">
+        <v>7167720</v>
+      </c>
+      <c r="L489" s="5" t="n">
+        <v>17148</v>
       </c>
       <c r="M489" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N489" s="3" t="inlineStr">
@@ -33570,22 +33182,18 @@
       </c>
       <c r="J491" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K491" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L491" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K491" s="5" t="n">
+        <v>5364240</v>
+      </c>
+      <c r="L491" s="5" t="n">
+        <v>17530</v>
       </c>
       <c r="M491" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N491" s="3" t="inlineStr">
@@ -33770,22 +33378,18 @@
       </c>
       <c r="J494" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K494" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L494" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K494" s="5" t="n">
+        <v>7947240</v>
+      </c>
+      <c r="L494" s="5" t="n">
+        <v>16696</v>
       </c>
       <c r="M494" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N494" s="3" t="inlineStr">
@@ -33902,22 +33506,18 @@
       </c>
       <c r="J496" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K496" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L496" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K496" s="5" t="n">
+        <v>7408800</v>
+      </c>
+      <c r="L496" s="5" t="n">
+        <v>16538</v>
       </c>
       <c r="M496" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N496" s="3" t="inlineStr">
@@ -33966,22 +33566,18 @@
       </c>
       <c r="J497" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K497" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L497" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K497" s="5" t="n">
+        <v>6987960</v>
+      </c>
+      <c r="L497" s="5" t="n">
+        <v>16718</v>
       </c>
       <c r="M497" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N497" s="3" t="inlineStr">
@@ -34098,22 +33694,18 @@
       </c>
       <c r="J499" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K499" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
-      </c>
-      <c r="L499" s="3" t="inlineStr">
-        <is>
-          <t>暂无</t>
-        </is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="K499" s="5" t="n">
+        <v>5297880</v>
+      </c>
+      <c r="L499" s="5" t="n">
+        <v>17313</v>
       </c>
       <c r="M499" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>90 天現金付款計劃</t>
         </is>
       </c>
       <c r="N499" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix: Synchronize exact HKP API list prices and sqft prices for 叡璟I open-for-sale units
</commit_message>
<xml_diff>
--- a/files/九龙-深水埗-叡璟I.xlsx
+++ b/files/九龙-深水埗-叡璟I.xlsx
@@ -4770,10 +4770,10 @@
         </is>
       </c>
       <c r="H62" s="5" t="n">
-        <v>727000</v>
+        <v>14727000</v>
       </c>
       <c r="I62" s="5" t="n">
-        <v>484</v>
+        <v>22484</v>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
@@ -4781,10 +4781,10 @@
         </is>
       </c>
       <c r="K62" s="5" t="n">
-        <v>610680</v>
+        <v>12370680</v>
       </c>
       <c r="L62" s="5" t="n">
-        <v>932</v>
+        <v>18887</v>
       </c>
       <c r="M62" s="3" t="inlineStr">
         <is>
@@ -5102,10 +5102,10 @@
         </is>
       </c>
       <c r="H67" s="5" t="n">
-        <v>683000</v>
+        <v>14683000</v>
       </c>
       <c r="I67" s="5" t="n">
-        <v>417</v>
+        <v>22417</v>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
@@ -5113,10 +5113,10 @@
         </is>
       </c>
       <c r="K67" s="5" t="n">
-        <v>573720</v>
+        <v>12333720</v>
       </c>
       <c r="L67" s="5" t="n">
-        <v>876</v>
+        <v>18830</v>
       </c>
       <c r="M67" s="3" t="inlineStr">
         <is>
@@ -5434,10 +5434,10 @@
         </is>
       </c>
       <c r="H72" s="5" t="n">
-        <v>639000</v>
+        <v>14639000</v>
       </c>
       <c r="I72" s="5" t="n">
-        <v>350</v>
+        <v>22350</v>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
@@ -5445,10 +5445,10 @@
         </is>
       </c>
       <c r="K72" s="5" t="n">
-        <v>536760</v>
+        <v>12296760</v>
       </c>
       <c r="L72" s="5" t="n">
-        <v>819</v>
+        <v>18774</v>
       </c>
       <c r="M72" s="3" t="inlineStr">
         <is>
@@ -5766,10 +5766,10 @@
         </is>
       </c>
       <c r="H77" s="5" t="n">
-        <v>595000</v>
+        <v>14595000</v>
       </c>
       <c r="I77" s="5" t="n">
-        <v>282</v>
+        <v>22282</v>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
@@ -5777,10 +5777,10 @@
         </is>
       </c>
       <c r="K77" s="5" t="n">
-        <v>499800</v>
+        <v>12259800</v>
       </c>
       <c r="L77" s="5" t="n">
-        <v>763</v>
+        <v>18717</v>
       </c>
       <c r="M77" s="3" t="inlineStr">
         <is>
@@ -6098,10 +6098,10 @@
         </is>
       </c>
       <c r="H82" s="5" t="n">
-        <v>552000</v>
+        <v>14552000</v>
       </c>
       <c r="I82" s="5" t="n">
-        <v>217</v>
+        <v>22217</v>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
@@ -6109,10 +6109,10 @@
         </is>
       </c>
       <c r="K82" s="5" t="n">
-        <v>463680</v>
+        <v>12223680</v>
       </c>
       <c r="L82" s="5" t="n">
-        <v>708</v>
+        <v>18662</v>
       </c>
       <c r="M82" s="3" t="inlineStr">
         <is>
@@ -6430,10 +6430,10 @@
         </is>
       </c>
       <c r="H87" s="5" t="n">
-        <v>508000</v>
+        <v>14508000</v>
       </c>
       <c r="I87" s="5" t="n">
-        <v>150</v>
+        <v>22150</v>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
@@ -6441,10 +6441,10 @@
         </is>
       </c>
       <c r="K87" s="5" t="n">
-        <v>426720</v>
+        <v>12186720</v>
       </c>
       <c r="L87" s="5" t="n">
-        <v>651</v>
+        <v>18606</v>
       </c>
       <c r="M87" s="3" t="inlineStr">
         <is>
@@ -6762,10 +6762,10 @@
         </is>
       </c>
       <c r="H92" s="5" t="n">
-        <v>465000</v>
+        <v>14465000</v>
       </c>
       <c r="I92" s="5" t="n">
-        <v>84</v>
+        <v>22084</v>
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
@@ -6773,10 +6773,10 @@
         </is>
       </c>
       <c r="K92" s="5" t="n">
-        <v>390600</v>
+        <v>12150600</v>
       </c>
       <c r="L92" s="5" t="n">
-        <v>596</v>
+        <v>18551</v>
       </c>
       <c r="M92" s="3" t="inlineStr">
         <is>
@@ -7094,10 +7094,10 @@
         </is>
       </c>
       <c r="H97" s="5" t="n">
-        <v>465000</v>
+        <v>14465000</v>
       </c>
       <c r="I97" s="5" t="n">
-        <v>84</v>
+        <v>22084</v>
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
@@ -7105,10 +7105,10 @@
         </is>
       </c>
       <c r="K97" s="5" t="n">
-        <v>390600</v>
+        <v>12150600</v>
       </c>
       <c r="L97" s="5" t="n">
-        <v>596</v>
+        <v>18551</v>
       </c>
       <c r="M97" s="3" t="inlineStr">
         <is>
@@ -7426,10 +7426,10 @@
         </is>
       </c>
       <c r="H102" s="5" t="n">
-        <v>379000</v>
+        <v>14379000</v>
       </c>
       <c r="I102" s="5" t="n">
-        <v>953</v>
+        <v>21953</v>
       </c>
       <c r="J102" s="3" t="inlineStr">
         <is>
@@ -7437,10 +7437,10 @@
         </is>
       </c>
       <c r="K102" s="5" t="n">
-        <v>318360</v>
+        <v>12078360</v>
       </c>
       <c r="L102" s="5" t="n">
-        <v>486</v>
+        <v>18440</v>
       </c>
       <c r="M102" s="3" t="inlineStr">
         <is>
@@ -8778,10 +8778,10 @@
         </is>
       </c>
       <c r="H122" s="5" t="n">
-        <v>193000</v>
+        <v>14193000</v>
       </c>
       <c r="I122" s="5" t="n">
-        <v>603</v>
+        <v>21603</v>
       </c>
       <c r="J122" s="3" t="inlineStr">
         <is>
@@ -8789,10 +8789,10 @@
         </is>
       </c>
       <c r="K122" s="5" t="n">
-        <v>162120</v>
+        <v>11922120</v>
       </c>
       <c r="L122" s="5" t="n">
-        <v>247</v>
+        <v>18146</v>
       </c>
       <c r="M122" s="3" t="inlineStr">
         <is>
@@ -9110,10 +9110,10 @@
         </is>
       </c>
       <c r="H127" s="5" t="n">
-        <v>164000</v>
+        <v>14164000</v>
       </c>
       <c r="I127" s="5" t="n">
-        <v>559</v>
+        <v>21559</v>
       </c>
       <c r="J127" s="3" t="inlineStr">
         <is>
@@ -9121,10 +9121,10 @@
         </is>
       </c>
       <c r="K127" s="5" t="n">
-        <v>137760</v>
+        <v>11897760</v>
       </c>
       <c r="L127" s="5" t="n">
-        <v>210</v>
+        <v>18109</v>
       </c>
       <c r="M127" s="3" t="inlineStr">
         <is>
@@ -9442,10 +9442,10 @@
         </is>
       </c>
       <c r="H132" s="5" t="n">
-        <v>136000</v>
+        <v>14136000</v>
       </c>
       <c r="I132" s="5" t="n">
-        <v>516</v>
+        <v>21516</v>
       </c>
       <c r="J132" s="3" t="inlineStr">
         <is>
@@ -9453,10 +9453,10 @@
         </is>
       </c>
       <c r="K132" s="5" t="n">
-        <v>114240</v>
+        <v>11874240</v>
       </c>
       <c r="L132" s="5" t="n">
-        <v>174</v>
+        <v>18073</v>
       </c>
       <c r="M132" s="3" t="inlineStr">
         <is>
@@ -9842,10 +9842,10 @@
         </is>
       </c>
       <c r="H138" s="5" t="n">
-        <v>10000</v>
+        <v>9010000</v>
       </c>
       <c r="I138" s="5" t="n">
-        <v>351</v>
+        <v>21351</v>
       </c>
       <c r="J138" s="3" t="inlineStr">
         <is>
@@ -9853,10 +9853,10 @@
         </is>
       </c>
       <c r="K138" s="5" t="n">
-        <v>8400</v>
+        <v>7568400</v>
       </c>
       <c r="L138" s="5" t="n">
-        <v>20</v>
+        <v>17935</v>
       </c>
       <c r="M138" s="3" t="inlineStr">
         <is>
@@ -10174,10 +10174,10 @@
         </is>
       </c>
       <c r="H143" s="5" t="n">
-        <v>983000</v>
+        <v>8983000</v>
       </c>
       <c r="I143" s="5" t="n">
-        <v>287</v>
+        <v>21287</v>
       </c>
       <c r="J143" s="3" t="inlineStr">
         <is>
@@ -10185,10 +10185,10 @@
         </is>
       </c>
       <c r="K143" s="5" t="n">
-        <v>825720</v>
+        <v>7545720</v>
       </c>
       <c r="L143" s="5" t="n">
-        <v>1957</v>
+        <v>17881</v>
       </c>
       <c r="M143" s="3" t="inlineStr">
         <is>
@@ -10506,10 +10506,10 @@
         </is>
       </c>
       <c r="H148" s="5" t="n">
-        <v>956000</v>
+        <v>8956000</v>
       </c>
       <c r="I148" s="5" t="n">
-        <v>223</v>
+        <v>21223</v>
       </c>
       <c r="J148" s="3" t="inlineStr">
         <is>
@@ -10517,10 +10517,10 @@
         </is>
       </c>
       <c r="K148" s="5" t="n">
-        <v>803040</v>
+        <v>7523040</v>
       </c>
       <c r="L148" s="5" t="n">
-        <v>1903</v>
+        <v>17827</v>
       </c>
       <c r="M148" s="3" t="inlineStr">
         <is>
@@ -10770,10 +10770,10 @@
         </is>
       </c>
       <c r="H152" s="5" t="n">
-        <v>23000</v>
+        <v>14023000</v>
       </c>
       <c r="I152" s="5" t="n">
-        <v>344</v>
+        <v>21344</v>
       </c>
       <c r="J152" s="3" t="inlineStr">
         <is>
@@ -10781,10 +10781,10 @@
         </is>
       </c>
       <c r="K152" s="5" t="n">
-        <v>19320</v>
+        <v>11779320</v>
       </c>
       <c r="L152" s="5" t="n">
-        <v>29</v>
+        <v>17929</v>
       </c>
       <c r="M152" s="3" t="inlineStr">
         <is>
@@ -10830,10 +10830,10 @@
         </is>
       </c>
       <c r="H153" s="5" t="n">
-        <v>911000</v>
+        <v>8911000</v>
       </c>
       <c r="I153" s="5" t="n">
-        <v>116</v>
+        <v>21116</v>
       </c>
       <c r="J153" s="3" t="inlineStr">
         <is>
@@ -10841,10 +10841,10 @@
         </is>
       </c>
       <c r="K153" s="5" t="n">
-        <v>765240</v>
+        <v>7485240</v>
       </c>
       <c r="L153" s="5" t="n">
-        <v>1813</v>
+        <v>17738</v>
       </c>
       <c r="M153" s="3" t="inlineStr">
         <is>
@@ -11094,10 +11094,10 @@
         </is>
       </c>
       <c r="H157" s="5" t="n">
-        <v>995000</v>
+        <v>13995000</v>
       </c>
       <c r="I157" s="5" t="n">
-        <v>301</v>
+        <v>21301</v>
       </c>
       <c r="J157" s="3" t="inlineStr">
         <is>
@@ -11105,10 +11105,10 @@
         </is>
       </c>
       <c r="K157" s="5" t="n">
-        <v>835800</v>
+        <v>11755800</v>
       </c>
       <c r="L157" s="5" t="n">
-        <v>1272</v>
+        <v>17893</v>
       </c>
       <c r="M157" s="3" t="inlineStr">
         <is>
@@ -11154,10 +11154,10 @@
         </is>
       </c>
       <c r="H158" s="5" t="n">
-        <v>849000</v>
+        <v>8849000</v>
       </c>
       <c r="I158" s="5" t="n">
-        <v>969</v>
+        <v>20969</v>
       </c>
       <c r="J158" s="3" t="inlineStr">
         <is>
@@ -11165,10 +11165,10 @@
         </is>
       </c>
       <c r="K158" s="5" t="n">
-        <v>713160</v>
+        <v>7433160</v>
       </c>
       <c r="L158" s="5" t="n">
-        <v>1690</v>
+        <v>17614</v>
       </c>
       <c r="M158" s="3" t="inlineStr">
         <is>
@@ -11418,10 +11418,10 @@
         </is>
       </c>
       <c r="H162" s="5" t="n">
-        <v>967000</v>
+        <v>13967000</v>
       </c>
       <c r="I162" s="5" t="n">
-        <v>259</v>
+        <v>21259</v>
       </c>
       <c r="J162" s="3" t="inlineStr">
         <is>
@@ -11429,10 +11429,10 @@
         </is>
       </c>
       <c r="K162" s="5" t="n">
-        <v>812280</v>
+        <v>11732280</v>
       </c>
       <c r="L162" s="5" t="n">
-        <v>1236</v>
+        <v>17857</v>
       </c>
       <c r="M162" s="3" t="inlineStr">
         <is>
@@ -11478,10 +11478,10 @@
         </is>
       </c>
       <c r="H163" s="5" t="n">
-        <v>716000</v>
+        <v>8716000</v>
       </c>
       <c r="I163" s="5" t="n">
-        <v>654</v>
+        <v>20654</v>
       </c>
       <c r="J163" s="3" t="inlineStr">
         <is>
@@ -11489,10 +11489,10 @@
         </is>
       </c>
       <c r="K163" s="5" t="n">
-        <v>601440</v>
+        <v>7321440</v>
       </c>
       <c r="L163" s="5" t="n">
-        <v>1425</v>
+        <v>17349</v>
       </c>
       <c r="M163" s="3" t="inlineStr">
         <is>
@@ -11810,10 +11810,10 @@
         </is>
       </c>
       <c r="H168" s="5" t="n">
-        <v>498000</v>
+        <v>8498000</v>
       </c>
       <c r="I168" s="5" t="n">
-        <v>137</v>
+        <v>20137</v>
       </c>
       <c r="J168" s="3" t="inlineStr">
         <is>
@@ -11821,10 +11821,10 @@
         </is>
       </c>
       <c r="K168" s="5" t="n">
-        <v>418320</v>
+        <v>7138320</v>
       </c>
       <c r="L168" s="5" t="n">
-        <v>991</v>
+        <v>16915</v>
       </c>
       <c r="M168" s="3" t="inlineStr">
         <is>
@@ -12142,10 +12142,10 @@
         </is>
       </c>
       <c r="H173" s="5" t="n">
-        <v>498000</v>
+        <v>8498000</v>
       </c>
       <c r="I173" s="5" t="n">
-        <v>137</v>
+        <v>20137</v>
       </c>
       <c r="J173" s="3" t="inlineStr">
         <is>
@@ -12153,10 +12153,10 @@
         </is>
       </c>
       <c r="K173" s="5" t="n">
-        <v>418320</v>
+        <v>7138320</v>
       </c>
       <c r="L173" s="5" t="n">
-        <v>991</v>
+        <v>16915</v>
       </c>
       <c r="M173" s="3" t="inlineStr">
         <is>
@@ -12474,10 +12474,10 @@
         </is>
       </c>
       <c r="H178" s="5" t="n">
-        <v>447000</v>
+        <v>8447000</v>
       </c>
       <c r="I178" s="5" t="n">
-        <v>17</v>
+        <v>20017</v>
       </c>
       <c r="J178" s="3" t="inlineStr">
         <is>
@@ -12485,10 +12485,10 @@
         </is>
       </c>
       <c r="K178" s="5" t="n">
-        <v>375480</v>
+        <v>7095480</v>
       </c>
       <c r="L178" s="5" t="n">
-        <v>890</v>
+        <v>16814</v>
       </c>
       <c r="M178" s="3" t="inlineStr">
         <is>
@@ -12738,10 +12738,10 @@
         </is>
       </c>
       <c r="H182" s="5" t="n">
-        <v>856000</v>
+        <v>13856000</v>
       </c>
       <c r="I182" s="5" t="n">
-        <v>90</v>
+        <v>21090</v>
       </c>
       <c r="J182" s="3" t="inlineStr">
         <is>
@@ -12749,10 +12749,10 @@
         </is>
       </c>
       <c r="K182" s="5" t="n">
-        <v>719040</v>
+        <v>11639040</v>
       </c>
       <c r="L182" s="5" t="n">
-        <v>1094</v>
+        <v>17715</v>
       </c>
       <c r="M182" s="3" t="inlineStr">
         <is>
@@ -12798,10 +12798,10 @@
         </is>
       </c>
       <c r="H183" s="5" t="n">
-        <v>422000</v>
+        <v>8422000</v>
       </c>
       <c r="I183" s="5" t="n">
-        <v>957</v>
+        <v>19957</v>
       </c>
       <c r="J183" s="3" t="inlineStr">
         <is>
@@ -12809,10 +12809,10 @@
         </is>
       </c>
       <c r="K183" s="5" t="n">
-        <v>354480</v>
+        <v>7074480</v>
       </c>
       <c r="L183" s="5" t="n">
-        <v>840</v>
+        <v>16764</v>
       </c>
       <c r="M183" s="3" t="inlineStr">
         <is>
@@ -13062,10 +13062,10 @@
         </is>
       </c>
       <c r="H187" s="5" t="n">
-        <v>828000</v>
+        <v>13828000</v>
       </c>
       <c r="I187" s="5" t="n">
-        <v>47</v>
+        <v>21047</v>
       </c>
       <c r="J187" s="3" t="inlineStr">
         <is>
@@ -13073,10 +13073,10 @@
         </is>
       </c>
       <c r="K187" s="5" t="n">
-        <v>695520</v>
+        <v>11615520</v>
       </c>
       <c r="L187" s="5" t="n">
-        <v>1059</v>
+        <v>17680</v>
       </c>
       <c r="M187" s="3" t="inlineStr">
         <is>
@@ -13122,10 +13122,10 @@
         </is>
       </c>
       <c r="H188" s="5" t="n">
-        <v>372000</v>
+        <v>8372000</v>
       </c>
       <c r="I188" s="5" t="n">
-        <v>839</v>
+        <v>19839</v>
       </c>
       <c r="J188" s="3" t="inlineStr">
         <is>
@@ -13133,10 +13133,10 @@
         </is>
       </c>
       <c r="K188" s="5" t="n">
-        <v>312480</v>
+        <v>7032480</v>
       </c>
       <c r="L188" s="5" t="n">
-        <v>740</v>
+        <v>16665</v>
       </c>
       <c r="M188" s="3" t="inlineStr">
         <is>
@@ -13386,10 +13386,10 @@
         </is>
       </c>
       <c r="H192" s="5" t="n">
-        <v>818000</v>
+        <v>13818000</v>
       </c>
       <c r="I192" s="5" t="n">
-        <v>32</v>
+        <v>21032</v>
       </c>
       <c r="J192" s="3" t="inlineStr">
         <is>
@@ -13397,10 +13397,10 @@
         </is>
       </c>
       <c r="K192" s="5" t="n">
-        <v>687120</v>
+        <v>11607120</v>
       </c>
       <c r="L192" s="5" t="n">
-        <v>1046</v>
+        <v>17667</v>
       </c>
       <c r="M192" s="3" t="inlineStr">
         <is>
@@ -15622,10 +15622,10 @@
         </is>
       </c>
       <c r="H225" s="5" t="n">
-        <v>322000</v>
+        <v>9322000</v>
       </c>
       <c r="I225" s="5" t="n">
-        <v>301</v>
+        <v>22301</v>
       </c>
       <c r="J225" s="3" t="inlineStr">
         <is>
@@ -15633,10 +15633,10 @@
         </is>
       </c>
       <c r="K225" s="5" t="n">
-        <v>270480</v>
+        <v>7830480</v>
       </c>
       <c r="L225" s="5" t="n">
-        <v>647</v>
+        <v>18733</v>
       </c>
       <c r="M225" s="3" t="inlineStr">
         <is>
@@ -16158,10 +16158,10 @@
         </is>
       </c>
       <c r="H233" s="5" t="n">
-        <v>295000</v>
+        <v>9295000</v>
       </c>
       <c r="I233" s="5" t="n">
-        <v>237</v>
+        <v>22237</v>
       </c>
       <c r="J233" s="3" t="inlineStr">
         <is>
@@ -16169,10 +16169,10 @@
         </is>
       </c>
       <c r="K233" s="5" t="n">
-        <v>247800</v>
+        <v>7807800</v>
       </c>
       <c r="L233" s="5" t="n">
-        <v>593</v>
+        <v>18679</v>
       </c>
       <c r="M233" s="3" t="inlineStr">
         <is>
@@ -16694,10 +16694,10 @@
         </is>
       </c>
       <c r="H241" s="5" t="n">
-        <v>267000</v>
+        <v>9267000</v>
       </c>
       <c r="I241" s="5" t="n">
-        <v>170</v>
+        <v>22170</v>
       </c>
       <c r="J241" s="3" t="inlineStr">
         <is>
@@ -16705,10 +16705,10 @@
         </is>
       </c>
       <c r="K241" s="5" t="n">
-        <v>224280</v>
+        <v>7784280</v>
       </c>
       <c r="L241" s="5" t="n">
-        <v>537</v>
+        <v>18623</v>
       </c>
       <c r="M241" s="3" t="inlineStr">
         <is>
@@ -17230,10 +17230,10 @@
         </is>
       </c>
       <c r="H249" s="5" t="n">
-        <v>239000</v>
+        <v>9239000</v>
       </c>
       <c r="I249" s="5" t="n">
-        <v>103</v>
+        <v>22103</v>
       </c>
       <c r="J249" s="3" t="inlineStr">
         <is>
@@ -17241,10 +17241,10 @@
         </is>
       </c>
       <c r="K249" s="5" t="n">
-        <v>200760</v>
+        <v>7760760</v>
       </c>
       <c r="L249" s="5" t="n">
-        <v>480</v>
+        <v>18566</v>
       </c>
       <c r="M249" s="3" t="inlineStr">
         <is>
@@ -17766,10 +17766,10 @@
         </is>
       </c>
       <c r="H257" s="5" t="n">
-        <v>211000</v>
+        <v>9211000</v>
       </c>
       <c r="I257" s="5" t="n">
-        <v>36</v>
+        <v>22036</v>
       </c>
       <c r="J257" s="3" t="inlineStr">
         <is>
@@ -17777,10 +17777,10 @@
         </is>
       </c>
       <c r="K257" s="5" t="n">
-        <v>177240</v>
+        <v>7737240</v>
       </c>
       <c r="L257" s="5" t="n">
-        <v>424</v>
+        <v>18510</v>
       </c>
       <c r="M257" s="3" t="inlineStr">
         <is>
@@ -18302,10 +18302,10 @@
         </is>
       </c>
       <c r="H265" s="5" t="n">
-        <v>184000</v>
+        <v>9184000</v>
       </c>
       <c r="I265" s="5" t="n">
-        <v>971</v>
+        <v>21971</v>
       </c>
       <c r="J265" s="3" t="inlineStr">
         <is>
@@ -18313,10 +18313,10 @@
         </is>
       </c>
       <c r="K265" s="5" t="n">
-        <v>154560</v>
+        <v>7714560</v>
       </c>
       <c r="L265" s="5" t="n">
-        <v>370</v>
+        <v>18456</v>
       </c>
       <c r="M265" s="3" t="inlineStr">
         <is>
@@ -18838,10 +18838,10 @@
         </is>
       </c>
       <c r="H273" s="5" t="n">
-        <v>184000</v>
+        <v>9184000</v>
       </c>
       <c r="I273" s="5" t="n">
-        <v>971</v>
+        <v>21971</v>
       </c>
       <c r="J273" s="3" t="inlineStr">
         <is>
@@ -18849,10 +18849,10 @@
         </is>
       </c>
       <c r="K273" s="5" t="n">
-        <v>154560</v>
+        <v>7714560</v>
       </c>
       <c r="L273" s="5" t="n">
-        <v>370</v>
+        <v>18456</v>
       </c>
       <c r="M273" s="3" t="inlineStr">
         <is>
@@ -19374,10 +19374,10 @@
         </is>
       </c>
       <c r="H281" s="5" t="n">
-        <v>129000</v>
+        <v>9129000</v>
       </c>
       <c r="I281" s="5" t="n">
-        <v>840</v>
+        <v>21840</v>
       </c>
       <c r="J281" s="3" t="inlineStr">
         <is>
@@ -19385,10 +19385,10 @@
         </is>
       </c>
       <c r="K281" s="5" t="n">
-        <v>108360</v>
+        <v>7668360</v>
       </c>
       <c r="L281" s="5" t="n">
-        <v>259</v>
+        <v>18345</v>
       </c>
       <c r="M281" s="3" t="inlineStr">
         <is>
@@ -19910,10 +19910,10 @@
         </is>
       </c>
       <c r="H289" s="5" t="n">
-        <v>102000</v>
+        <v>9102000</v>
       </c>
       <c r="I289" s="5" t="n">
-        <v>775</v>
+        <v>21775</v>
       </c>
       <c r="J289" s="3" t="inlineStr">
         <is>
@@ -19921,10 +19921,10 @@
         </is>
       </c>
       <c r="K289" s="5" t="n">
-        <v>85680</v>
+        <v>7645680</v>
       </c>
       <c r="L289" s="5" t="n">
-        <v>205</v>
+        <v>18291</v>
       </c>
       <c r="M289" s="3" t="inlineStr">
         <is>
@@ -20038,10 +20038,10 @@
         </is>
       </c>
       <c r="H291" s="5" t="n">
-        <v>27000</v>
+        <v>7027000</v>
       </c>
       <c r="I291" s="5" t="n">
-        <v>964</v>
+        <v>22964</v>
       </c>
       <c r="J291" s="3" t="inlineStr">
         <is>
@@ -20049,10 +20049,10 @@
         </is>
       </c>
       <c r="K291" s="5" t="n">
-        <v>22680</v>
+        <v>5902680</v>
       </c>
       <c r="L291" s="5" t="n">
-        <v>74</v>
+        <v>19290</v>
       </c>
       <c r="M291" s="3" t="inlineStr">
         <is>
@@ -20438,10 +20438,10 @@
         </is>
       </c>
       <c r="H297" s="5" t="n">
-        <v>75000</v>
+        <v>9075000</v>
       </c>
       <c r="I297" s="5" t="n">
-        <v>711</v>
+        <v>21711</v>
       </c>
       <c r="J297" s="3" t="inlineStr">
         <is>
@@ -20449,10 +20449,10 @@
         </is>
       </c>
       <c r="K297" s="5" t="n">
-        <v>63000</v>
+        <v>7623000</v>
       </c>
       <c r="L297" s="5" t="n">
-        <v>151</v>
+        <v>18237</v>
       </c>
       <c r="M297" s="3" t="inlineStr">
         <is>
@@ -20566,10 +20566,10 @@
         </is>
       </c>
       <c r="H299" s="5" t="n">
-        <v>6000</v>
+        <v>7006000</v>
       </c>
       <c r="I299" s="5" t="n">
-        <v>895</v>
+        <v>22895</v>
       </c>
       <c r="J299" s="3" t="inlineStr">
         <is>
@@ -20577,10 +20577,10 @@
         </is>
       </c>
       <c r="K299" s="5" t="n">
-        <v>5040</v>
+        <v>5885040</v>
       </c>
       <c r="L299" s="5" t="n">
-        <v>16</v>
+        <v>19232</v>
       </c>
       <c r="M299" s="3" t="inlineStr">
         <is>
@@ -20966,10 +20966,10 @@
         </is>
       </c>
       <c r="H305" s="5" t="n">
-        <v>47000</v>
+        <v>9047000</v>
       </c>
       <c r="I305" s="5" t="n">
-        <v>644</v>
+        <v>21644</v>
       </c>
       <c r="J305" s="3" t="inlineStr">
         <is>
@@ -20977,10 +20977,10 @@
         </is>
       </c>
       <c r="K305" s="5" t="n">
-        <v>39480</v>
+        <v>7599480</v>
       </c>
       <c r="L305" s="5" t="n">
-        <v>94</v>
+        <v>18181</v>
       </c>
       <c r="M305" s="3" t="inlineStr">
         <is>
@@ -21094,10 +21094,10 @@
         </is>
       </c>
       <c r="H307" s="5" t="n">
-        <v>985000</v>
+        <v>6985000</v>
       </c>
       <c r="I307" s="5" t="n">
-        <v>827</v>
+        <v>22827</v>
       </c>
       <c r="J307" s="3" t="inlineStr">
         <is>
@@ -21105,10 +21105,10 @@
         </is>
       </c>
       <c r="K307" s="5" t="n">
-        <v>827400</v>
+        <v>5867400</v>
       </c>
       <c r="L307" s="5" t="n">
-        <v>2704</v>
+        <v>19175</v>
       </c>
       <c r="M307" s="3" t="inlineStr">
         <is>
@@ -21494,10 +21494,10 @@
         </is>
       </c>
       <c r="H313" s="5" t="n">
-        <v>20000</v>
+        <v>9020000</v>
       </c>
       <c r="I313" s="5" t="n">
-        <v>579</v>
+        <v>21579</v>
       </c>
       <c r="J313" s="3" t="inlineStr">
         <is>
@@ -21505,10 +21505,10 @@
         </is>
       </c>
       <c r="K313" s="5" t="n">
-        <v>16800</v>
+        <v>7576800</v>
       </c>
       <c r="L313" s="5" t="n">
-        <v>40</v>
+        <v>18126</v>
       </c>
       <c r="M313" s="3" t="inlineStr">
         <is>
@@ -21622,10 +21622,10 @@
         </is>
       </c>
       <c r="H315" s="5" t="n">
-        <v>964000</v>
+        <v>6964000</v>
       </c>
       <c r="I315" s="5" t="n">
-        <v>758</v>
+        <v>22758</v>
       </c>
       <c r="J315" s="3" t="inlineStr">
         <is>
@@ -21633,10 +21633,10 @@
         </is>
       </c>
       <c r="K315" s="5" t="n">
-        <v>809760</v>
+        <v>5849760</v>
       </c>
       <c r="L315" s="5" t="n">
-        <v>2646</v>
+        <v>19117</v>
       </c>
       <c r="M315" s="3" t="inlineStr">
         <is>
@@ -22022,10 +22022,10 @@
         </is>
       </c>
       <c r="H321" s="5" t="n">
-        <v>993000</v>
+        <v>8993000</v>
       </c>
       <c r="I321" s="5" t="n">
-        <v>514</v>
+        <v>21514</v>
       </c>
       <c r="J321" s="3" t="inlineStr">
         <is>
@@ -22033,10 +22033,10 @@
         </is>
       </c>
       <c r="K321" s="5" t="n">
-        <v>834120</v>
+        <v>7554120</v>
       </c>
       <c r="L321" s="5" t="n">
-        <v>1996</v>
+        <v>18072</v>
       </c>
       <c r="M321" s="3" t="inlineStr">
         <is>
@@ -22150,10 +22150,10 @@
         </is>
       </c>
       <c r="H323" s="5" t="n">
-        <v>943000</v>
+        <v>6943000</v>
       </c>
       <c r="I323" s="5" t="n">
-        <v>690</v>
+        <v>22690</v>
       </c>
       <c r="J323" s="3" t="inlineStr">
         <is>
@@ -22161,10 +22161,10 @@
         </is>
       </c>
       <c r="K323" s="5" t="n">
-        <v>792120</v>
+        <v>5832120</v>
       </c>
       <c r="L323" s="5" t="n">
-        <v>2589</v>
+        <v>19059</v>
       </c>
       <c r="M323" s="3" t="inlineStr">
         <is>
@@ -22550,10 +22550,10 @@
         </is>
       </c>
       <c r="H329" s="5" t="n">
-        <v>966000</v>
+        <v>8966000</v>
       </c>
       <c r="I329" s="5" t="n">
-        <v>450</v>
+        <v>21450</v>
       </c>
       <c r="J329" s="3" t="inlineStr">
         <is>
@@ -22561,10 +22561,10 @@
         </is>
       </c>
       <c r="K329" s="5" t="n">
-        <v>811440</v>
+        <v>7531440</v>
       </c>
       <c r="L329" s="5" t="n">
-        <v>1941</v>
+        <v>18018</v>
       </c>
       <c r="M329" s="3" t="inlineStr">
         <is>
@@ -22678,10 +22678,10 @@
         </is>
       </c>
       <c r="H331" s="5" t="n">
-        <v>922000</v>
+        <v>6922000</v>
       </c>
       <c r="I331" s="5" t="n">
-        <v>621</v>
+        <v>22621</v>
       </c>
       <c r="J331" s="3" t="inlineStr">
         <is>
@@ -22689,10 +22689,10 @@
         </is>
       </c>
       <c r="K331" s="5" t="n">
-        <v>774480</v>
+        <v>5814480</v>
       </c>
       <c r="L331" s="5" t="n">
-        <v>2531</v>
+        <v>19002</v>
       </c>
       <c r="M331" s="3" t="inlineStr">
         <is>
@@ -23078,10 +23078,10 @@
         </is>
       </c>
       <c r="H337" s="5" t="n">
-        <v>940000</v>
+        <v>8940000</v>
       </c>
       <c r="I337" s="5" t="n">
-        <v>388</v>
+        <v>21388</v>
       </c>
       <c r="J337" s="3" t="inlineStr">
         <is>
@@ -23089,10 +23089,10 @@
         </is>
       </c>
       <c r="K337" s="5" t="n">
-        <v>789600</v>
+        <v>7509600</v>
       </c>
       <c r="L337" s="5" t="n">
-        <v>1889</v>
+        <v>17966</v>
       </c>
       <c r="M337" s="3" t="inlineStr">
         <is>
@@ -23206,10 +23206,10 @@
         </is>
       </c>
       <c r="H339" s="5" t="n">
-        <v>902000</v>
+        <v>6902000</v>
       </c>
       <c r="I339" s="5" t="n">
-        <v>556</v>
+        <v>22556</v>
       </c>
       <c r="J339" s="3" t="inlineStr">
         <is>
@@ -23217,10 +23217,10 @@
         </is>
       </c>
       <c r="K339" s="5" t="n">
-        <v>757680</v>
+        <v>5797680</v>
       </c>
       <c r="L339" s="5" t="n">
-        <v>2476</v>
+        <v>18947</v>
       </c>
       <c r="M339" s="3" t="inlineStr">
         <is>
@@ -23606,10 +23606,10 @@
         </is>
       </c>
       <c r="H345" s="5" t="n">
-        <v>940000</v>
+        <v>8940000</v>
       </c>
       <c r="I345" s="5" t="n">
-        <v>388</v>
+        <v>21388</v>
       </c>
       <c r="J345" s="3" t="inlineStr">
         <is>
@@ -23617,10 +23617,10 @@
         </is>
       </c>
       <c r="K345" s="5" t="n">
-        <v>789600</v>
+        <v>7509600</v>
       </c>
       <c r="L345" s="5" t="n">
-        <v>1889</v>
+        <v>17966</v>
       </c>
       <c r="M345" s="3" t="inlineStr">
         <is>
@@ -23734,10 +23734,10 @@
         </is>
       </c>
       <c r="H347" s="5" t="n">
-        <v>902000</v>
+        <v>6902000</v>
       </c>
       <c r="I347" s="5" t="n">
-        <v>556</v>
+        <v>22556</v>
       </c>
       <c r="J347" s="3" t="inlineStr">
         <is>
@@ -23745,10 +23745,10 @@
         </is>
       </c>
       <c r="K347" s="5" t="n">
-        <v>757680</v>
+        <v>5797680</v>
       </c>
       <c r="L347" s="5" t="n">
-        <v>2476</v>
+        <v>18947</v>
       </c>
       <c r="M347" s="3" t="inlineStr">
         <is>
@@ -24134,10 +24134,10 @@
         </is>
       </c>
       <c r="H353" s="5" t="n">
-        <v>886000</v>
+        <v>8886000</v>
       </c>
       <c r="I353" s="5" t="n">
-        <v>258</v>
+        <v>21258</v>
       </c>
       <c r="J353" s="3" t="inlineStr">
         <is>
@@ -24145,10 +24145,10 @@
         </is>
       </c>
       <c r="K353" s="5" t="n">
-        <v>744240</v>
+        <v>7464240</v>
       </c>
       <c r="L353" s="5" t="n">
-        <v>1780</v>
+        <v>17857</v>
       </c>
       <c r="M353" s="3" t="inlineStr">
         <is>
@@ -24262,10 +24262,10 @@
         </is>
       </c>
       <c r="H355" s="5" t="n">
-        <v>861000</v>
+        <v>6861000</v>
       </c>
       <c r="I355" s="5" t="n">
-        <v>422</v>
+        <v>22422</v>
       </c>
       <c r="J355" s="3" t="inlineStr">
         <is>
@@ -24273,10 +24273,10 @@
         </is>
       </c>
       <c r="K355" s="5" t="n">
-        <v>723240</v>
+        <v>5763240</v>
       </c>
       <c r="L355" s="5" t="n">
-        <v>2364</v>
+        <v>18834</v>
       </c>
       <c r="M355" s="3" t="inlineStr">
         <is>
@@ -24662,10 +24662,10 @@
         </is>
       </c>
       <c r="H361" s="5" t="n">
-        <v>882000</v>
+        <v>8882000</v>
       </c>
       <c r="I361" s="5" t="n">
-        <v>47</v>
+        <v>21047</v>
       </c>
       <c r="J361" s="3" t="inlineStr">
         <is>
@@ -24673,10 +24673,10 @@
         </is>
       </c>
       <c r="K361" s="5" t="n">
-        <v>740880</v>
+        <v>7460880</v>
       </c>
       <c r="L361" s="5" t="n">
-        <v>1756</v>
+        <v>17680</v>
       </c>
       <c r="M361" s="3" t="inlineStr">
         <is>
@@ -25198,10 +25198,10 @@
         </is>
       </c>
       <c r="H369" s="5" t="n">
-        <v>864000</v>
+        <v>8864000</v>
       </c>
       <c r="I369" s="5" t="n">
-        <v>5</v>
+        <v>21005</v>
       </c>
       <c r="J369" s="3" t="inlineStr">
         <is>
@@ -25209,10 +25209,10 @@
         </is>
       </c>
       <c r="K369" s="5" t="n">
-        <v>725760</v>
+        <v>7445760</v>
       </c>
       <c r="L369" s="5" t="n">
-        <v>1720</v>
+        <v>17644</v>
       </c>
       <c r="M369" s="3" t="inlineStr">
         <is>
@@ -25734,10 +25734,10 @@
         </is>
       </c>
       <c r="H377" s="5" t="n">
-        <v>846000</v>
+        <v>8846000</v>
       </c>
       <c r="I377" s="5" t="n">
-        <v>962</v>
+        <v>20962</v>
       </c>
       <c r="J377" s="3" t="inlineStr">
         <is>
@@ -25745,10 +25745,10 @@
         </is>
       </c>
       <c r="K377" s="5" t="n">
-        <v>710640</v>
+        <v>7430640</v>
       </c>
       <c r="L377" s="5" t="n">
-        <v>1684</v>
+        <v>17608</v>
       </c>
       <c r="M377" s="3" t="inlineStr">
         <is>
@@ -26066,10 +26066,10 @@
         </is>
       </c>
       <c r="H382" s="5" t="n">
-        <v>306000</v>
+        <v>10306000</v>
       </c>
       <c r="I382" s="5" t="n">
-        <v>651</v>
+        <v>21651</v>
       </c>
       <c r="J382" s="3" t="inlineStr">
         <is>
@@ -26077,10 +26077,10 @@
         </is>
       </c>
       <c r="K382" s="5" t="n">
-        <v>257040</v>
+        <v>8657040</v>
       </c>
       <c r="L382" s="5" t="n">
-        <v>540</v>
+        <v>18187</v>
       </c>
       <c r="M382" s="3" t="inlineStr">
         <is>
@@ -26262,10 +26262,10 @@
         </is>
       </c>
       <c r="H385" s="5" t="n">
-        <v>828000</v>
+        <v>8828000</v>
       </c>
       <c r="I385" s="5" t="n">
-        <v>919</v>
+        <v>20919</v>
       </c>
       <c r="J385" s="3" t="inlineStr">
         <is>
@@ -26273,10 +26273,10 @@
         </is>
       </c>
       <c r="K385" s="5" t="n">
-        <v>695520</v>
+        <v>7415520</v>
       </c>
       <c r="L385" s="5" t="n">
-        <v>1648</v>
+        <v>17572</v>
       </c>
       <c r="M385" s="3" t="inlineStr">
         <is>
@@ -26390,10 +26390,10 @@
         </is>
       </c>
       <c r="H387" s="5" t="n">
-        <v>687000</v>
+        <v>6687000</v>
       </c>
       <c r="I387" s="5" t="n">
-        <v>997</v>
+        <v>21997</v>
       </c>
       <c r="J387" s="3" t="inlineStr">
         <is>
@@ -26401,10 +26401,10 @@
         </is>
       </c>
       <c r="K387" s="5" t="n">
-        <v>577080</v>
+        <v>5617080</v>
       </c>
       <c r="L387" s="5" t="n">
-        <v>1898</v>
+        <v>18477</v>
       </c>
       <c r="M387" s="3" t="inlineStr">
         <is>
@@ -26586,10 +26586,10 @@
         </is>
       </c>
       <c r="H390" s="5" t="n">
-        <v>275000</v>
+        <v>10275000</v>
       </c>
       <c r="I390" s="5" t="n">
-        <v>586</v>
+        <v>21586</v>
       </c>
       <c r="J390" s="3" t="inlineStr">
         <is>
@@ -26597,10 +26597,10 @@
         </is>
       </c>
       <c r="K390" s="5" t="n">
-        <v>231000</v>
+        <v>8631000</v>
       </c>
       <c r="L390" s="5" t="n">
-        <v>485</v>
+        <v>18132</v>
       </c>
       <c r="M390" s="3" t="inlineStr">
         <is>
@@ -26782,10 +26782,10 @@
         </is>
       </c>
       <c r="H393" s="5" t="n">
-        <v>811000</v>
+        <v>8811000</v>
       </c>
       <c r="I393" s="5" t="n">
-        <v>879</v>
+        <v>20879</v>
       </c>
       <c r="J393" s="3" t="inlineStr">
         <is>
@@ -26793,10 +26793,10 @@
         </is>
       </c>
       <c r="K393" s="5" t="n">
-        <v>681240</v>
+        <v>7401240</v>
       </c>
       <c r="L393" s="5" t="n">
-        <v>1614</v>
+        <v>17538</v>
       </c>
       <c r="M393" s="3" t="inlineStr">
         <is>
@@ -26910,10 +26910,10 @@
         </is>
       </c>
       <c r="H395" s="5" t="n">
-        <v>667000</v>
+        <v>6667000</v>
       </c>
       <c r="I395" s="5" t="n">
-        <v>931</v>
+        <v>21931</v>
       </c>
       <c r="J395" s="3" t="inlineStr">
         <is>
@@ -26921,10 +26921,10 @@
         </is>
       </c>
       <c r="K395" s="5" t="n">
-        <v>560280</v>
+        <v>5600280</v>
       </c>
       <c r="L395" s="5" t="n">
-        <v>1843</v>
+        <v>18422</v>
       </c>
       <c r="M395" s="3" t="inlineStr">
         <is>
@@ -27106,10 +27106,10 @@
         </is>
       </c>
       <c r="H398" s="5" t="n">
-        <v>244000</v>
+        <v>10244000</v>
       </c>
       <c r="I398" s="5" t="n">
-        <v>521</v>
+        <v>21521</v>
       </c>
       <c r="J398" s="3" t="inlineStr">
         <is>
@@ -27117,10 +27117,10 @@
         </is>
       </c>
       <c r="K398" s="5" t="n">
-        <v>204960</v>
+        <v>8604960</v>
       </c>
       <c r="L398" s="5" t="n">
-        <v>431</v>
+        <v>18078</v>
       </c>
       <c r="M398" s="3" t="inlineStr">
         <is>
@@ -27302,10 +27302,10 @@
         </is>
       </c>
       <c r="H401" s="5" t="n">
-        <v>793000</v>
+        <v>8793000</v>
       </c>
       <c r="I401" s="5" t="n">
-        <v>836</v>
+        <v>20836</v>
       </c>
       <c r="J401" s="3" t="inlineStr">
         <is>
@@ -27313,10 +27313,10 @@
         </is>
       </c>
       <c r="K401" s="5" t="n">
-        <v>666120</v>
+        <v>7386120</v>
       </c>
       <c r="L401" s="5" t="n">
-        <v>1578</v>
+        <v>17503</v>
       </c>
       <c r="M401" s="3" t="inlineStr">
         <is>
@@ -27430,10 +27430,10 @@
         </is>
       </c>
       <c r="H403" s="5" t="n">
-        <v>647000</v>
+        <v>6647000</v>
       </c>
       <c r="I403" s="5" t="n">
-        <v>865</v>
+        <v>21865</v>
       </c>
       <c r="J403" s="3" t="inlineStr">
         <is>
@@ -27441,10 +27441,10 @@
         </is>
       </c>
       <c r="K403" s="5" t="n">
-        <v>543480</v>
+        <v>5583480</v>
       </c>
       <c r="L403" s="5" t="n">
-        <v>1788</v>
+        <v>18367</v>
       </c>
       <c r="M403" s="3" t="inlineStr">
         <is>
@@ -27830,10 +27830,10 @@
         </is>
       </c>
       <c r="H409" s="5" t="n">
-        <v>793000</v>
+        <v>8793000</v>
       </c>
       <c r="I409" s="5" t="n">
-        <v>836</v>
+        <v>20836</v>
       </c>
       <c r="J409" s="3" t="inlineStr">
         <is>
@@ -27841,10 +27841,10 @@
         </is>
       </c>
       <c r="K409" s="5" t="n">
-        <v>666120</v>
+        <v>7386120</v>
       </c>
       <c r="L409" s="5" t="n">
-        <v>1578</v>
+        <v>17503</v>
       </c>
       <c r="M409" s="3" t="inlineStr">
         <is>
@@ -28298,10 +28298,10 @@
         </is>
       </c>
       <c r="H416" s="5" t="n">
-        <v>494000</v>
+        <v>9494000</v>
       </c>
       <c r="I416" s="5" t="n">
-        <v>192</v>
+        <v>21192</v>
       </c>
       <c r="J416" s="3" t="inlineStr">
         <is>
@@ -28309,10 +28309,10 @@
         </is>
       </c>
       <c r="K416" s="5" t="n">
-        <v>414960</v>
+        <v>7974960</v>
       </c>
       <c r="L416" s="5" t="n">
-        <v>926</v>
+        <v>17801</v>
       </c>
       <c r="M416" s="3" t="inlineStr">
         <is>
@@ -28358,10 +28358,10 @@
         </is>
       </c>
       <c r="H417" s="5" t="n">
-        <v>758000</v>
+        <v>8758000</v>
       </c>
       <c r="I417" s="5" t="n">
-        <v>754</v>
+        <v>20754</v>
       </c>
       <c r="J417" s="3" t="inlineStr">
         <is>
@@ -28369,10 +28369,10 @@
         </is>
       </c>
       <c r="K417" s="5" t="n">
-        <v>636720</v>
+        <v>7356720</v>
       </c>
       <c r="L417" s="5" t="n">
-        <v>1509</v>
+        <v>17433</v>
       </c>
       <c r="M417" s="3" t="inlineStr">
         <is>
@@ -28826,10 +28826,10 @@
         </is>
       </c>
       <c r="H424" s="5" t="n">
-        <v>466000</v>
+        <v>9466000</v>
       </c>
       <c r="I424" s="5" t="n">
-        <v>129</v>
+        <v>21129</v>
       </c>
       <c r="J424" s="3" t="inlineStr">
         <is>
@@ -28837,10 +28837,10 @@
         </is>
       </c>
       <c r="K424" s="5" t="n">
-        <v>391440</v>
+        <v>7951440</v>
       </c>
       <c r="L424" s="5" t="n">
-        <v>874</v>
+        <v>17749</v>
       </c>
       <c r="M424" s="3" t="inlineStr">
         <is>
@@ -28886,10 +28886,10 @@
         </is>
       </c>
       <c r="H425" s="5" t="n">
-        <v>741000</v>
+        <v>8741000</v>
       </c>
       <c r="I425" s="5" t="n">
-        <v>713</v>
+        <v>20713</v>
       </c>
       <c r="J425" s="3" t="inlineStr">
         <is>
@@ -28897,10 +28897,10 @@
         </is>
       </c>
       <c r="K425" s="5" t="n">
-        <v>622440</v>
+        <v>7342440</v>
       </c>
       <c r="L425" s="5" t="n">
-        <v>1475</v>
+        <v>17399</v>
       </c>
       <c r="M425" s="3" t="inlineStr">
         <is>
@@ -29218,10 +29218,10 @@
         </is>
       </c>
       <c r="H430" s="5" t="n">
-        <v>122000</v>
+        <v>10122000</v>
       </c>
       <c r="I430" s="5" t="n">
-        <v>265</v>
+        <v>21265</v>
       </c>
       <c r="J430" s="3" t="inlineStr">
         <is>
@@ -29229,10 +29229,10 @@
         </is>
       </c>
       <c r="K430" s="5" t="n">
-        <v>102480</v>
+        <v>8502480</v>
       </c>
       <c r="L430" s="5" t="n">
-        <v>215</v>
+        <v>17862</v>
       </c>
       <c r="M430" s="3" t="inlineStr">
         <is>
@@ -29346,10 +29346,10 @@
         </is>
       </c>
       <c r="H432" s="5" t="n">
-        <v>438000</v>
+        <v>9438000</v>
       </c>
       <c r="I432" s="5" t="n">
-        <v>67</v>
+        <v>21067</v>
       </c>
       <c r="J432" s="3" t="inlineStr">
         <is>
@@ -29357,10 +29357,10 @@
         </is>
       </c>
       <c r="K432" s="5" t="n">
-        <v>367920</v>
+        <v>7927920</v>
       </c>
       <c r="L432" s="5" t="n">
-        <v>821</v>
+        <v>17696</v>
       </c>
       <c r="M432" s="3" t="inlineStr">
         <is>
@@ -29406,10 +29406,10 @@
         </is>
       </c>
       <c r="H433" s="5" t="n">
-        <v>723000</v>
+        <v>8723000</v>
       </c>
       <c r="I433" s="5" t="n">
-        <v>671</v>
+        <v>20671</v>
       </c>
       <c r="J433" s="3" t="inlineStr">
         <is>
@@ -29417,10 +29417,10 @@
         </is>
       </c>
       <c r="K433" s="5" t="n">
-        <v>607320</v>
+        <v>7327320</v>
       </c>
       <c r="L433" s="5" t="n">
-        <v>1439</v>
+        <v>17363</v>
       </c>
       <c r="M433" s="3" t="inlineStr">
         <is>
@@ -29534,10 +29534,10 @@
         </is>
       </c>
       <c r="H435" s="5" t="n">
-        <v>567000</v>
+        <v>6567000</v>
       </c>
       <c r="I435" s="5" t="n">
-        <v>602</v>
+        <v>21602</v>
       </c>
       <c r="J435" s="3" t="inlineStr">
         <is>
@@ -29545,10 +29545,10 @@
         </is>
       </c>
       <c r="K435" s="5" t="n">
-        <v>476280</v>
+        <v>5516280</v>
       </c>
       <c r="L435" s="5" t="n">
-        <v>1567</v>
+        <v>18146</v>
       </c>
       <c r="M435" s="3" t="inlineStr">
         <is>
@@ -29730,10 +29730,10 @@
         </is>
       </c>
       <c r="H438" s="5" t="n">
-        <v>71000</v>
+        <v>10071000</v>
       </c>
       <c r="I438" s="5" t="n">
-        <v>158</v>
+        <v>21158</v>
       </c>
       <c r="J438" s="3" t="inlineStr">
         <is>
@@ -29741,10 +29741,10 @@
         </is>
       </c>
       <c r="K438" s="5" t="n">
-        <v>59640</v>
+        <v>8459640</v>
       </c>
       <c r="L438" s="5" t="n">
-        <v>125</v>
+        <v>17772</v>
       </c>
       <c r="M438" s="3" t="inlineStr">
         <is>
@@ -29858,10 +29858,10 @@
         </is>
       </c>
       <c r="H440" s="5" t="n">
-        <v>390000</v>
+        <v>9390000</v>
       </c>
       <c r="I440" s="5" t="n">
-        <v>960</v>
+        <v>20960</v>
       </c>
       <c r="J440" s="3" t="inlineStr">
         <is>
@@ -29869,10 +29869,10 @@
         </is>
       </c>
       <c r="K440" s="5" t="n">
-        <v>327600</v>
+        <v>7887600</v>
       </c>
       <c r="L440" s="5" t="n">
-        <v>731</v>
+        <v>17606</v>
       </c>
       <c r="M440" s="3" t="inlineStr">
         <is>
@@ -29918,10 +29918,10 @@
         </is>
       </c>
       <c r="H441" s="5" t="n">
-        <v>706000</v>
+        <v>8706000</v>
       </c>
       <c r="I441" s="5" t="n">
-        <v>630</v>
+        <v>20630</v>
       </c>
       <c r="J441" s="3" t="inlineStr">
         <is>
@@ -29929,10 +29929,10 @@
         </is>
       </c>
       <c r="K441" s="5" t="n">
-        <v>593040</v>
+        <v>7313040</v>
       </c>
       <c r="L441" s="5" t="n">
-        <v>1405</v>
+        <v>17329</v>
       </c>
       <c r="M441" s="3" t="inlineStr">
         <is>
@@ -30046,10 +30046,10 @@
         </is>
       </c>
       <c r="H443" s="5" t="n">
-        <v>548000</v>
+        <v>6548000</v>
       </c>
       <c r="I443" s="5" t="n">
-        <v>539</v>
+        <v>21539</v>
       </c>
       <c r="J443" s="3" t="inlineStr">
         <is>
@@ -30057,10 +30057,10 @@
         </is>
       </c>
       <c r="K443" s="5" t="n">
-        <v>460320</v>
+        <v>5500320</v>
       </c>
       <c r="L443" s="5" t="n">
-        <v>1514</v>
+        <v>18093</v>
       </c>
       <c r="M443" s="3" t="inlineStr">
         <is>
@@ -30242,10 +30242,10 @@
         </is>
       </c>
       <c r="H446" s="5" t="n">
-        <v>1000</v>
+        <v>10001000</v>
       </c>
       <c r="I446" s="5" t="n">
-        <v>11</v>
+        <v>21011</v>
       </c>
       <c r="J446" s="3" t="inlineStr">
         <is>
@@ -30253,10 +30253,10 @@
         </is>
       </c>
       <c r="K446" s="5" t="n">
-        <v>840</v>
+        <v>8400840</v>
       </c>
       <c r="L446" s="5" t="n">
-        <v>2</v>
+        <v>17649</v>
       </c>
       <c r="M446" s="3" t="inlineStr">
         <is>
@@ -30370,10 +30370,10 @@
         </is>
       </c>
       <c r="H448" s="5" t="n">
-        <v>325000</v>
+        <v>9325000</v>
       </c>
       <c r="I448" s="5" t="n">
-        <v>815</v>
+        <v>20815</v>
       </c>
       <c r="J448" s="3" t="inlineStr">
         <is>
@@ -30381,10 +30381,10 @@
         </is>
       </c>
       <c r="K448" s="5" t="n">
-        <v>273000</v>
+        <v>7833000</v>
       </c>
       <c r="L448" s="5" t="n">
-        <v>609</v>
+        <v>17484</v>
       </c>
       <c r="M448" s="3" t="inlineStr">
         <is>
@@ -30430,10 +30430,10 @@
         </is>
       </c>
       <c r="H449" s="5" t="n">
-        <v>688000</v>
+        <v>8688000</v>
       </c>
       <c r="I449" s="5" t="n">
-        <v>588</v>
+        <v>20588</v>
       </c>
       <c r="J449" s="3" t="inlineStr">
         <is>
@@ -30441,10 +30441,10 @@
         </is>
       </c>
       <c r="K449" s="5" t="n">
-        <v>577920</v>
+        <v>7297920</v>
       </c>
       <c r="L449" s="5" t="n">
-        <v>1369</v>
+        <v>17294</v>
       </c>
       <c r="M449" s="3" t="inlineStr">
         <is>
@@ -30558,10 +30558,10 @@
         </is>
       </c>
       <c r="H451" s="5" t="n">
-        <v>528000</v>
+        <v>6528000</v>
       </c>
       <c r="I451" s="5" t="n">
-        <v>474</v>
+        <v>21474</v>
       </c>
       <c r="J451" s="3" t="inlineStr">
         <is>
@@ -30569,10 +30569,10 @@
         </is>
       </c>
       <c r="K451" s="5" t="n">
-        <v>443520</v>
+        <v>5483520</v>
       </c>
       <c r="L451" s="5" t="n">
-        <v>1459</v>
+        <v>18038</v>
       </c>
       <c r="M451" s="3" t="inlineStr">
         <is>
@@ -30890,10 +30890,10 @@
         </is>
       </c>
       <c r="H456" s="5" t="n">
-        <v>185000</v>
+        <v>9185000</v>
       </c>
       <c r="I456" s="5" t="n">
-        <v>502</v>
+        <v>20502</v>
       </c>
       <c r="J456" s="3" t="inlineStr">
         <is>
@@ -30901,10 +30901,10 @@
         </is>
       </c>
       <c r="K456" s="5" t="n">
-        <v>155400</v>
+        <v>7715400</v>
       </c>
       <c r="L456" s="5" t="n">
-        <v>347</v>
+        <v>17222</v>
       </c>
       <c r="M456" s="3" t="inlineStr">
         <is>
@@ -30950,10 +30950,10 @@
         </is>
       </c>
       <c r="H457" s="5" t="n">
-        <v>671000</v>
+        <v>8671000</v>
       </c>
       <c r="I457" s="5" t="n">
-        <v>547</v>
+        <v>20547</v>
       </c>
       <c r="J457" s="3" t="inlineStr">
         <is>
@@ -30961,10 +30961,10 @@
         </is>
       </c>
       <c r="K457" s="5" t="n">
-        <v>563640</v>
+        <v>7283640</v>
       </c>
       <c r="L457" s="5" t="n">
-        <v>1336</v>
+        <v>17260</v>
       </c>
       <c r="M457" s="3" t="inlineStr">
         <is>
@@ -31418,10 +31418,10 @@
         </is>
       </c>
       <c r="H464" s="5" t="n">
-        <v>955000</v>
+        <v>8955000</v>
       </c>
       <c r="I464" s="5" t="n">
-        <v>989</v>
+        <v>19989</v>
       </c>
       <c r="J464" s="3" t="inlineStr">
         <is>
@@ -31429,10 +31429,10 @@
         </is>
       </c>
       <c r="K464" s="5" t="n">
-        <v>802200</v>
+        <v>7522200</v>
       </c>
       <c r="L464" s="5" t="n">
-        <v>1791</v>
+        <v>16791</v>
       </c>
       <c r="M464" s="3" t="inlineStr">
         <is>
@@ -31478,10 +31478,10 @@
         </is>
       </c>
       <c r="H465" s="5" t="n">
-        <v>653000</v>
+        <v>8653000</v>
       </c>
       <c r="I465" s="5" t="n">
-        <v>505</v>
+        <v>20505</v>
       </c>
       <c r="J465" s="3" t="inlineStr">
         <is>
@@ -31489,10 +31489,10 @@
         </is>
       </c>
       <c r="K465" s="5" t="n">
-        <v>548520</v>
+        <v>7268520</v>
       </c>
       <c r="L465" s="5" t="n">
-        <v>1300</v>
+        <v>17224</v>
       </c>
       <c r="M465" s="3" t="inlineStr">
         <is>
@@ -31946,10 +31946,10 @@
         </is>
       </c>
       <c r="H472" s="5" t="n">
-        <v>955000</v>
+        <v>8955000</v>
       </c>
       <c r="I472" s="5" t="n">
-        <v>989</v>
+        <v>19989</v>
       </c>
       <c r="J472" s="3" t="inlineStr">
         <is>
@@ -31957,10 +31957,10 @@
         </is>
       </c>
       <c r="K472" s="5" t="n">
-        <v>802200</v>
+        <v>7522200</v>
       </c>
       <c r="L472" s="5" t="n">
-        <v>1791</v>
+        <v>16791</v>
       </c>
       <c r="M472" s="3" t="inlineStr">
         <is>
@@ -32006,10 +32006,10 @@
         </is>
       </c>
       <c r="H473" s="5" t="n">
-        <v>653000</v>
+        <v>8653000</v>
       </c>
       <c r="I473" s="5" t="n">
-        <v>505</v>
+        <v>20505</v>
       </c>
       <c r="J473" s="3" t="inlineStr">
         <is>
@@ -32017,10 +32017,10 @@
         </is>
       </c>
       <c r="K473" s="5" t="n">
-        <v>548520</v>
+        <v>7268520</v>
       </c>
       <c r="L473" s="5" t="n">
-        <v>1300</v>
+        <v>17224</v>
       </c>
       <c r="M473" s="3" t="inlineStr">
         <is>
@@ -32338,10 +32338,10 @@
         </is>
       </c>
       <c r="H478" s="5" t="n">
-        <v>547000</v>
+        <v>9547000</v>
       </c>
       <c r="I478" s="5" t="n">
-        <v>57</v>
+        <v>20057</v>
       </c>
       <c r="J478" s="3" t="inlineStr">
         <is>
@@ -32349,10 +32349,10 @@
         </is>
       </c>
       <c r="K478" s="5" t="n">
-        <v>459480</v>
+        <v>8019480</v>
       </c>
       <c r="L478" s="5" t="n">
-        <v>965</v>
+        <v>16848</v>
       </c>
       <c r="M478" s="3" t="inlineStr">
         <is>
@@ -32466,10 +32466,10 @@
         </is>
       </c>
       <c r="H480" s="5" t="n">
-        <v>901000</v>
+        <v>8901000</v>
       </c>
       <c r="I480" s="5" t="n">
-        <v>868</v>
+        <v>19868</v>
       </c>
       <c r="J480" s="3" t="inlineStr">
         <is>
@@ -32477,10 +32477,10 @@
         </is>
       </c>
       <c r="K480" s="5" t="n">
-        <v>756840</v>
+        <v>7476840</v>
       </c>
       <c r="L480" s="5" t="n">
-        <v>1689</v>
+        <v>16689</v>
       </c>
       <c r="M480" s="3" t="inlineStr">
         <is>
@@ -32526,10 +32526,10 @@
         </is>
       </c>
       <c r="H481" s="5" t="n">
-        <v>619000</v>
+        <v>8619000</v>
       </c>
       <c r="I481" s="5" t="n">
-        <v>424</v>
+        <v>20424</v>
       </c>
       <c r="J481" s="3" t="inlineStr">
         <is>
@@ -32537,10 +32537,10 @@
         </is>
       </c>
       <c r="K481" s="5" t="n">
-        <v>519960</v>
+        <v>7239960</v>
       </c>
       <c r="L481" s="5" t="n">
-        <v>1232</v>
+        <v>17156</v>
       </c>
       <c r="M481" s="3" t="inlineStr">
         <is>
@@ -32654,10 +32654,10 @@
         </is>
       </c>
       <c r="H483" s="5" t="n">
-        <v>450000</v>
+        <v>6450000</v>
       </c>
       <c r="I483" s="5" t="n">
-        <v>217</v>
+        <v>21217</v>
       </c>
       <c r="J483" s="3" t="inlineStr">
         <is>
@@ -32665,10 +32665,10 @@
         </is>
       </c>
       <c r="K483" s="5" t="n">
-        <v>378000</v>
+        <v>5418000</v>
       </c>
       <c r="L483" s="5" t="n">
-        <v>1243</v>
+        <v>17822</v>
       </c>
       <c r="M483" s="3" t="inlineStr">
         <is>
@@ -32850,10 +32850,10 @@
         </is>
       </c>
       <c r="H486" s="5" t="n">
-        <v>518000</v>
+        <v>9518000</v>
       </c>
       <c r="I486" s="5" t="n">
-        <v>996</v>
+        <v>19996</v>
       </c>
       <c r="J486" s="3" t="inlineStr">
         <is>
@@ -32861,10 +32861,10 @@
         </is>
       </c>
       <c r="K486" s="5" t="n">
-        <v>435120</v>
+        <v>7995120</v>
       </c>
       <c r="L486" s="5" t="n">
-        <v>914</v>
+        <v>16796</v>
       </c>
       <c r="M486" s="3" t="inlineStr">
         <is>
@@ -32978,10 +32978,10 @@
         </is>
       </c>
       <c r="H488" s="5" t="n">
-        <v>875000</v>
+        <v>8875000</v>
       </c>
       <c r="I488" s="5" t="n">
-        <v>810</v>
+        <v>19810</v>
       </c>
       <c r="J488" s="3" t="inlineStr">
         <is>
@@ -32989,10 +32989,10 @@
         </is>
       </c>
       <c r="K488" s="5" t="n">
-        <v>735000</v>
+        <v>7455000</v>
       </c>
       <c r="L488" s="5" t="n">
-        <v>1641</v>
+        <v>16641</v>
       </c>
       <c r="M488" s="3" t="inlineStr">
         <is>
@@ -33038,10 +33038,10 @@
         </is>
       </c>
       <c r="H489" s="5" t="n">
-        <v>533000</v>
+        <v>8533000</v>
       </c>
       <c r="I489" s="5" t="n">
-        <v>220</v>
+        <v>20220</v>
       </c>
       <c r="J489" s="3" t="inlineStr">
         <is>
@@ -33049,10 +33049,10 @@
         </is>
       </c>
       <c r="K489" s="5" t="n">
-        <v>447720</v>
+        <v>7167720</v>
       </c>
       <c r="L489" s="5" t="n">
-        <v>1061</v>
+        <v>16985</v>
       </c>
       <c r="M489" s="3" t="inlineStr">
         <is>
@@ -33166,10 +33166,10 @@
         </is>
       </c>
       <c r="H491" s="5" t="n">
-        <v>386000</v>
+        <v>6386000</v>
       </c>
       <c r="I491" s="5" t="n">
-        <v>7</v>
+        <v>21007</v>
       </c>
       <c r="J491" s="3" t="inlineStr">
         <is>
@@ -33177,10 +33177,10 @@
         </is>
       </c>
       <c r="K491" s="5" t="n">
-        <v>324240</v>
+        <v>5364240</v>
       </c>
       <c r="L491" s="5" t="n">
-        <v>1067</v>
+        <v>17646</v>
       </c>
       <c r="M491" s="3" t="inlineStr">
         <is>
@@ -33362,10 +33362,10 @@
         </is>
       </c>
       <c r="H494" s="5" t="n">
-        <v>461000</v>
+        <v>9461000</v>
       </c>
       <c r="I494" s="5" t="n">
-        <v>876</v>
+        <v>19876</v>
       </c>
       <c r="J494" s="3" t="inlineStr">
         <is>
@@ -33373,10 +33373,10 @@
         </is>
       </c>
       <c r="K494" s="5" t="n">
-        <v>387240</v>
+        <v>7947240</v>
       </c>
       <c r="L494" s="5" t="n">
-        <v>814</v>
+        <v>16696</v>
       </c>
       <c r="M494" s="3" t="inlineStr">
         <is>
@@ -33490,10 +33490,10 @@
         </is>
       </c>
       <c r="H496" s="5" t="n">
-        <v>820000</v>
+        <v>8820000</v>
       </c>
       <c r="I496" s="5" t="n">
-        <v>688</v>
+        <v>19688</v>
       </c>
       <c r="J496" s="3" t="inlineStr">
         <is>
@@ -33501,10 +33501,10 @@
         </is>
       </c>
       <c r="K496" s="5" t="n">
-        <v>688800</v>
+        <v>7408800</v>
       </c>
       <c r="L496" s="5" t="n">
-        <v>1538</v>
+        <v>16538</v>
       </c>
       <c r="M496" s="3" t="inlineStr">
         <is>
@@ -33550,10 +33550,10 @@
         </is>
       </c>
       <c r="H497" s="5" t="n">
-        <v>319000</v>
+        <v>8319000</v>
       </c>
       <c r="I497" s="5" t="n">
-        <v>713</v>
+        <v>19713</v>
       </c>
       <c r="J497" s="3" t="inlineStr">
         <is>
@@ -33561,10 +33561,10 @@
         </is>
       </c>
       <c r="K497" s="5" t="n">
-        <v>267960</v>
+        <v>6987960</v>
       </c>
       <c r="L497" s="5" t="n">
-        <v>635</v>
+        <v>16559</v>
       </c>
       <c r="M497" s="3" t="inlineStr">
         <is>
@@ -33678,10 +33678,10 @@
         </is>
       </c>
       <c r="H499" s="5" t="n">
-        <v>307000</v>
+        <v>6307000</v>
       </c>
       <c r="I499" s="5" t="n">
-        <v>747</v>
+        <v>20747</v>
       </c>
       <c r="J499" s="3" t="inlineStr">
         <is>
@@ -33689,10 +33689,10 @@
         </is>
       </c>
       <c r="K499" s="5" t="n">
-        <v>257880</v>
+        <v>5297880</v>
       </c>
       <c r="L499" s="5" t="n">
-        <v>848</v>
+        <v>17427</v>
       </c>
       <c r="M499" s="3" t="inlineStr">
         <is>
@@ -35016,8 +35016,8 @@
       <c r="B16" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$73万
-$484/呎
+$1473万
+$22,484/呎
 (在售)</t>
         </is>
       </c>
@@ -35061,8 +35061,8 @@
       <c r="B17" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$68万
-$417/呎
+$1468万
+$22,417/呎
 (在售)</t>
         </is>
       </c>
@@ -35106,8 +35106,8 @@
       <c r="B18" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$64万
-$350/呎
+$1464万
+$22,350/呎
 (在售)</t>
         </is>
       </c>
@@ -35151,8 +35151,8 @@
       <c r="B19" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$60万
-$282/呎
+$1460万
+$22,282/呎
 (在售)</t>
         </is>
       </c>
@@ -35196,8 +35196,8 @@
       <c r="B20" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$55万
-$217/呎
+$1455万
+$22,217/呎
 (在售)</t>
         </is>
       </c>
@@ -35241,8 +35241,8 @@
       <c r="B21" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$51万
-$150/呎
+$1451万
+$22,150/呎
 (在售)</t>
         </is>
       </c>
@@ -35286,8 +35286,8 @@
       <c r="B22" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$46万
-$84/呎
+$1446万
+$22,084/呎
 (在售)</t>
         </is>
       </c>
@@ -35331,8 +35331,8 @@
       <c r="B23" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$46万
-$84/呎
+$1446万
+$22,084/呎
 (在售)</t>
         </is>
       </c>
@@ -35376,8 +35376,8 @@
       <c r="B24" s="21" t="inlineStr">
         <is>
           <t>A | 655呎 (3房1套)
-$38万
-$953/呎
+$1438万
+$21,953/呎
 (在售)</t>
         </is>
       </c>
@@ -35556,8 +35556,8 @@
       <c r="B28" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$19万
-$603/呎
+$1419万
+$21,603/呎
 (在售)</t>
         </is>
       </c>
@@ -35601,8 +35601,8 @@
       <c r="B29" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$16万
-$559/呎
+$1416万
+$21,559/呎
 (在售)</t>
         </is>
       </c>
@@ -35646,8 +35646,8 @@
       <c r="B30" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$14万
-$516/呎
+$1414万
+$21,516/呎
 (在售)</t>
         </is>
       </c>
@@ -35768,8 +35768,8 @@
       <c r="F32" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$1万
-$351/呎
+$901万
+$21,351/呎
 (在售)</t>
         </is>
       </c>
@@ -35813,8 +35813,8 @@
       <c r="F33" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$98万
-$287/呎
+$898万
+$21,287/呎
 (在售)</t>
         </is>
       </c>
@@ -35826,8 +35826,8 @@
       <c r="B34" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$2万
-$344/呎
+$1402万
+$21,344/呎
 (在售)</t>
         </is>
       </c>
@@ -35858,8 +35858,8 @@
       <c r="F34" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$96万
-$223/呎
+$896万
+$21,223/呎
 (在售)</t>
         </is>
       </c>
@@ -35871,8 +35871,8 @@
       <c r="B35" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$100万
-$301/呎
+$1400万
+$21,301/呎
 (在售)</t>
         </is>
       </c>
@@ -35903,8 +35903,8 @@
       <c r="F35" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$91万
-$116/呎
+$891万
+$21,116/呎
 (在售)</t>
         </is>
       </c>
@@ -35916,8 +35916,8 @@
       <c r="B36" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$97万
-$259/呎
+$1397万
+$21,259/呎
 (在售)</t>
         </is>
       </c>
@@ -35948,8 +35948,8 @@
       <c r="F36" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$85万
-$969/呎
+$885万
+$20,969/呎
 (在售)</t>
         </is>
       </c>
@@ -35993,8 +35993,8 @@
       <c r="F37" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$72万
-$654/呎
+$872万
+$20,654/呎
 (在售)</t>
         </is>
       </c>
@@ -36038,8 +36038,8 @@
       <c r="F38" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$50万
-$137/呎
+$850万
+$20,137/呎
 (在售)</t>
         </is>
       </c>
@@ -36083,8 +36083,8 @@
       <c r="F39" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$50万
-$137/呎
+$850万
+$20,137/呎
 (在售)</t>
         </is>
       </c>
@@ -36096,8 +36096,8 @@
       <c r="B40" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$86万
-$90/呎
+$1386万
+$21,090/呎
 (在售)</t>
         </is>
       </c>
@@ -36128,8 +36128,8 @@
       <c r="F40" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$45万
-$17/呎
+$845万
+$20,017/呎
 (在售)</t>
         </is>
       </c>
@@ -36141,8 +36141,8 @@
       <c r="B41" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$83万
-$47/呎
+$1383万
+$21,047/呎
 (在售)</t>
         </is>
       </c>
@@ -36173,8 +36173,8 @@
       <c r="F41" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$42万
-$957/呎
+$842万
+$19,957/呎
 (在售)</t>
         </is>
       </c>
@@ -36186,8 +36186,8 @@
       <c r="B42" s="21" t="inlineStr">
         <is>
           <t>A | 657呎 (3房1套)
-$82万
-$32/呎
+$1382万
+$21,032/呎
 (在售)</t>
         </is>
       </c>
@@ -36218,8 +36218,8 @@
       <c r="F42" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$37万
-$839/呎
+$837万
+$19,839/呎
 (在售)</t>
         </is>
       </c>
@@ -36662,8 +36662,8 @@
       <c r="F8" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$32万
-$301/呎
+$932万
+$22,301/呎
 (在售)</t>
         </is>
       </c>
@@ -36731,8 +36731,8 @@
       <c r="F9" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$30万
-$237/呎
+$930万
+$22,237/呎
 (在售)</t>
         </is>
       </c>
@@ -36800,8 +36800,8 @@
       <c r="F10" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$27万
-$170/呎
+$927万
+$22,170/呎
 (在售)</t>
         </is>
       </c>
@@ -36869,8 +36869,8 @@
       <c r="F11" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$24万
-$103/呎
+$924万
+$22,103/呎
 (在售)</t>
         </is>
       </c>
@@ -36938,8 +36938,8 @@
       <c r="F12" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$21万
-$36/呎
+$921万
+$22,036/呎
 (在售)</t>
         </is>
       </c>
@@ -37007,8 +37007,8 @@
       <c r="F13" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$18万
-$971/呎
+$918万
+$21,971/呎
 (在售)</t>
         </is>
       </c>
@@ -37076,8 +37076,8 @@
       <c r="F14" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$18万
-$971/呎
+$918万
+$21,971/呎
 (在售)</t>
         </is>
       </c>
@@ -37145,8 +37145,8 @@
       <c r="F15" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$13万
-$840/呎
+$913万
+$21,840/呎
 (在售)</t>
         </is>
       </c>
@@ -37198,8 +37198,8 @@
       <c r="D16" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$3万
-$964/呎
+$703万
+$22,964/呎
 (在售)</t>
         </is>
       </c>
@@ -37214,8 +37214,8 @@
       <c r="F16" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$10万
-$775/呎
+$910万
+$21,775/呎
 (在售)</t>
         </is>
       </c>
@@ -37267,8 +37267,8 @@
       <c r="D17" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$1万
-$895/呎
+$701万
+$22,895/呎
 (在售)</t>
         </is>
       </c>
@@ -37283,8 +37283,8 @@
       <c r="F17" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$8万
-$711/呎
+$908万
+$21,711/呎
 (在售)</t>
         </is>
       </c>
@@ -37336,8 +37336,8 @@
       <c r="D18" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$98万
-$827/呎
+$698万
+$22,827/呎
 (在售)</t>
         </is>
       </c>
@@ -37352,8 +37352,8 @@
       <c r="F18" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$5万
-$644/呎
+$905万
+$21,644/呎
 (在售)</t>
         </is>
       </c>
@@ -37405,8 +37405,8 @@
       <c r="D19" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$96万
-$758/呎
+$696万
+$22,758/呎
 (在售)</t>
         </is>
       </c>
@@ -37421,8 +37421,8 @@
       <c r="F19" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$2万
-$579/呎
+$902万
+$21,579/呎
 (在售)</t>
         </is>
       </c>
@@ -37474,8 +37474,8 @@
       <c r="D20" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$94万
-$690/呎
+$694万
+$22,690/呎
 (在售)</t>
         </is>
       </c>
@@ -37490,8 +37490,8 @@
       <c r="F20" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$99万
-$514/呎
+$899万
+$21,514/呎
 (在售)</t>
         </is>
       </c>
@@ -37543,8 +37543,8 @@
       <c r="D21" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$92万
-$621/呎
+$692万
+$22,621/呎
 (在售)</t>
         </is>
       </c>
@@ -37559,8 +37559,8 @@
       <c r="F21" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$97万
-$450/呎
+$897万
+$21,450/呎
 (在售)</t>
         </is>
       </c>
@@ -37612,8 +37612,8 @@
       <c r="D22" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$90万
-$556/呎
+$690万
+$22,556/呎
 (在售)</t>
         </is>
       </c>
@@ -37628,8 +37628,8 @@
       <c r="F22" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$94万
-$388/呎
+$894万
+$21,388/呎
 (在售)</t>
         </is>
       </c>
@@ -37681,8 +37681,8 @@
       <c r="D23" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$90万
-$556/呎
+$690万
+$22,556/呎
 (在售)</t>
         </is>
       </c>
@@ -37697,8 +37697,8 @@
       <c r="F23" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$94万
-$388/呎
+$894万
+$21,388/呎
 (在售)</t>
         </is>
       </c>
@@ -37750,8 +37750,8 @@
       <c r="D24" s="21" t="inlineStr">
         <is>
           <t>C | 306呎 (1房)
-$86万
-$422/呎
+$686万
+$22,422/呎
 (在售)</t>
         </is>
       </c>
@@ -37766,8 +37766,8 @@
       <c r="F24" s="21" t="inlineStr">
         <is>
           <t>E | 418呎 (2房)
-$89万
-$258/呎
+$889万
+$21,258/呎
 (在售)</t>
         </is>
       </c>
@@ -37835,8 +37835,8 @@
       <c r="F25" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$88万
-$47/呎
+$888万
+$21,047/呎
 (在售)</t>
         </is>
       </c>
@@ -37904,8 +37904,8 @@
       <c r="F26" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$86万
-$5/呎
+$886万
+$21,005/呎
 (在售)</t>
         </is>
       </c>
@@ -37973,8 +37973,8 @@
       <c r="F27" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$85万
-$962/呎
+$885万
+$20,962/呎
 (在售)</t>
         </is>
       </c>
@@ -38026,8 +38026,8 @@
       <c r="D28" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$69万
-$997/呎
+$669万
+$21,997/呎
 (在售)</t>
         </is>
       </c>
@@ -38042,8 +38042,8 @@
       <c r="F28" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$83万
-$919/呎
+$883万
+$20,919/呎
 (在售)</t>
         </is>
       </c>
@@ -38066,8 +38066,8 @@
       <c r="I28" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$31万
-$651/呎
+$1031万
+$21,651/呎
 (在售)</t>
         </is>
       </c>
@@ -38095,8 +38095,8 @@
       <c r="D29" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$67万
-$931/呎
+$667万
+$21,931/呎
 (在售)</t>
         </is>
       </c>
@@ -38111,8 +38111,8 @@
       <c r="F29" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$81万
-$879/呎
+$881万
+$20,879/呎
 (在售)</t>
         </is>
       </c>
@@ -38135,8 +38135,8 @@
       <c r="I29" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$28万
-$586/呎
+$1028万
+$21,586/呎
 (在售)</t>
         </is>
       </c>
@@ -38164,8 +38164,8 @@
       <c r="D30" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$65万
-$865/呎
+$665万
+$21,865/呎
 (在售)</t>
         </is>
       </c>
@@ -38180,8 +38180,8 @@
       <c r="F30" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$79万
-$836/呎
+$879万
+$20,836/呎
 (在售)</t>
         </is>
       </c>
@@ -38204,8 +38204,8 @@
       <c r="I30" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$24万
-$521/呎
+$1024万
+$21,521/呎
 (在售)</t>
         </is>
       </c>
@@ -38249,8 +38249,8 @@
       <c r="F31" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$79万
-$836/呎
+$879万
+$20,836/呎
 (在售)</t>
         </is>
       </c>
@@ -38318,16 +38318,16 @@
       <c r="F32" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$76万
-$754/呎
+$876万
+$20,754/呎
 (在售)</t>
         </is>
       </c>
       <c r="G32" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$49万
-$192/呎
+$949万
+$21,192/呎
 (在售)</t>
         </is>
       </c>
@@ -38387,16 +38387,16 @@
       <c r="F33" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$74万
-$713/呎
+$874万
+$20,713/呎
 (在售)</t>
         </is>
       </c>
       <c r="G33" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$47万
-$129/呎
+$947万
+$21,129/呎
 (在售)</t>
         </is>
       </c>
@@ -38440,8 +38440,8 @@
       <c r="D34" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$57万
-$602/呎
+$657万
+$21,602/呎
 (在售)</t>
         </is>
       </c>
@@ -38456,16 +38456,16 @@
       <c r="F34" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$72万
-$671/呎
+$872万
+$20,671/呎
 (在售)</t>
         </is>
       </c>
       <c r="G34" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$44万
-$67/呎
+$944万
+$21,067/呎
 (在售)</t>
         </is>
       </c>
@@ -38480,8 +38480,8 @@
       <c r="I34" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$12万
-$265/呎
+$1012万
+$21,265/呎
 (在售)</t>
         </is>
       </c>
@@ -38509,8 +38509,8 @@
       <c r="D35" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$55万
-$539/呎
+$655万
+$21,539/呎
 (在售)</t>
         </is>
       </c>
@@ -38525,16 +38525,16 @@
       <c r="F35" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$71万
-$630/呎
+$871万
+$20,630/呎
 (在售)</t>
         </is>
       </c>
       <c r="G35" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$39万
-$960/呎
+$939万
+$20,960/呎
 (在售)</t>
         </is>
       </c>
@@ -38549,8 +38549,8 @@
       <c r="I35" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$7万
-$158/呎
+$1007万
+$21,158/呎
 (在售)</t>
         </is>
       </c>
@@ -38578,8 +38578,8 @@
       <c r="D36" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$53万
-$474/呎
+$653万
+$21,474/呎
 (在售)</t>
         </is>
       </c>
@@ -38594,16 +38594,16 @@
       <c r="F36" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$69万
-$588/呎
+$869万
+$20,588/呎
 (在售)</t>
         </is>
       </c>
       <c r="G36" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$32万
-$815/呎
+$932万
+$20,815/呎
 (在售)</t>
         </is>
       </c>
@@ -38618,8 +38618,8 @@
       <c r="I36" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$0万
-$11/呎
+$1000万
+$21,011/呎
 (在售)</t>
         </is>
       </c>
@@ -38663,16 +38663,16 @@
       <c r="F37" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$67万
-$547/呎
+$867万
+$20,547/呎
 (在售)</t>
         </is>
       </c>
       <c r="G37" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$18万
-$502/呎
+$918万
+$20,502/呎
 (在售)</t>
         </is>
       </c>
@@ -38732,16 +38732,16 @@
       <c r="F38" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$65万
-$505/呎
+$865万
+$20,505/呎
 (在售)</t>
         </is>
       </c>
       <c r="G38" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$96万
-$989/呎
+$896万
+$19,989/呎
 (在售)</t>
         </is>
       </c>
@@ -38801,16 +38801,16 @@
       <c r="F39" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$65万
-$505/呎
+$865万
+$20,505/呎
 (在售)</t>
         </is>
       </c>
       <c r="G39" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$96万
-$989/呎
+$896万
+$19,989/呎
 (在售)</t>
         </is>
       </c>
@@ -38854,8 +38854,8 @@
       <c r="D40" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$45万
-$217/呎
+$645万
+$21,217/呎
 (在售)</t>
         </is>
       </c>
@@ -38870,16 +38870,16 @@
       <c r="F40" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$62万
-$424/呎
+$862万
+$20,424/呎
 (在售)</t>
         </is>
       </c>
       <c r="G40" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$90万
-$868/呎
+$890万
+$19,868/呎
 (在售)</t>
         </is>
       </c>
@@ -38894,8 +38894,8 @@
       <c r="I40" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$55万
-$57/呎
+$955万
+$20,057/呎
 (在售)</t>
         </is>
       </c>
@@ -38923,8 +38923,8 @@
       <c r="D41" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$39万
-$7/呎
+$639万
+$21,007/呎
 (在售)</t>
         </is>
       </c>
@@ -38939,16 +38939,16 @@
       <c r="F41" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$53万
-$220/呎
+$853万
+$20,220/呎
 (在售)</t>
         </is>
       </c>
       <c r="G41" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$88万
-$810/呎
+$888万
+$19,810/呎
 (在售)</t>
         </is>
       </c>
@@ -38963,8 +38963,8 @@
       <c r="I41" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$52万
-$996/呎
+$952万
+$19,996/呎
 (在售)</t>
         </is>
       </c>
@@ -38992,8 +38992,8 @@
       <c r="D42" s="21" t="inlineStr">
         <is>
           <t>C | 304呎 (1房)
-$31万
-$747/呎
+$631万
+$20,747/呎
 (在售)</t>
         </is>
       </c>
@@ -39008,16 +39008,16 @@
       <c r="F42" s="21" t="inlineStr">
         <is>
           <t>E | 422呎 (2房)
-$32万
-$713/呎
+$832万
+$19,713/呎
 (在售)</t>
         </is>
       </c>
       <c r="G42" s="21" t="inlineStr">
         <is>
           <t>F | 448呎 (2房)
-$82万
-$688/呎
+$882万
+$19,688/呎
 (在售)</t>
         </is>
       </c>
@@ -39032,8 +39032,8 @@
       <c r="I42" s="21" t="inlineStr">
         <is>
           <t>H | 476呎 (2房)
-$46万
-$876/呎
+$946万
+$19,876/呎
 (在售)</t>
         </is>
       </c>

</xml_diff>